<commit_message>
changes in the assessment page
</commit_message>
<xml_diff>
--- a/scratch/tracker.xlsx
+++ b/scratch/tracker.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30602"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30606"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://drpinnacle-my.sharepoint.com/personal/vish_drpinnacle_com/Documents/Projects/openvals/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3233" documentId="8_{F24D4BFB-FFC1-BD42-9143-22F6B790B9D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F832B7A0-A963-4D73-9C15-8703A49DA3BE}"/>
+  <xr:revisionPtr revIDLastSave="3264" documentId="8_{F24D4BFB-FFC1-BD42-9143-22F6B790B9D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B56F1BE5-F1B5-4FDC-9A77-6F61C3D3CFA2}"/>
   <bookViews>
     <workbookView xWindow="3960" yWindow="2780" windowWidth="28040" windowHeight="17180" xr2:uid="{BEF502B7-096A-F24C-A77D-ED0F5F38F7FE}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1081" uniqueCount="378">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1086" uniqueCount="380">
   <si>
     <t>Date</t>
   </si>
@@ -1176,6 +1176,12 @@
   </si>
   <si>
     <t>791 MB</t>
+  </si>
+  <si>
+    <t>qwen2-math:1.5b</t>
+  </si>
+  <si>
+    <t>935MB</t>
   </si>
 </sst>
 </file>
@@ -11347,35 +11353,63 @@
     </row>
     <row r="181" spans="1:22" ht="15.75" customHeight="1">
       <c r="A181" s="33">
-        <v>46304</v>
+        <v>46307</v>
       </c>
       <c r="B181" s="26" t="s">
         <v>367</v>
       </c>
-      <c r="C181" s="10"/>
-      <c r="D181" s="10"/>
-      <c r="E181" s="10"/>
-      <c r="F181" s="10"/>
+      <c r="C181" t="s">
+        <v>378</v>
+      </c>
+      <c r="D181" t="s">
+        <v>34</v>
+      </c>
+      <c r="E181" t="s">
+        <v>379</v>
+      </c>
+      <c r="F181" s="10" t="s">
+        <v>31</v>
+      </c>
       <c r="G181" s="10"/>
       <c r="H181" s="10"/>
       <c r="I181" s="10"/>
       <c r="J181" s="10"/>
       <c r="K181" s="10"/>
       <c r="L181" s="10"/>
-      <c r="M181" s="10"/>
+      <c r="M181" s="30"/>
       <c r="N181" s="10"/>
-      <c r="O181" s="10"/>
-      <c r="P181" s="10"/>
-      <c r="Q181" s="10"/>
-      <c r="R181" s="10"/>
-      <c r="S181" s="10"/>
-      <c r="T181" s="10"/>
-      <c r="U181" s="10"/>
-      <c r="V181" s="10"/>
+      <c r="O181" s="10">
+        <v>0.95</v>
+      </c>
+      <c r="P181" s="10">
+        <v>0.36199999999999999</v>
+      </c>
+      <c r="Q181" s="10">
+        <v>15537.3</v>
+      </c>
+      <c r="R181" s="10">
+        <v>0.48899999999999999</v>
+      </c>
+      <c r="S181" s="10">
+        <v>0.68200000000000005</v>
+      </c>
+      <c r="T181" s="10">
+        <v>1</v>
+      </c>
+      <c r="U181" s="10">
+        <v>0.92400000000000004</v>
+      </c>
+      <c r="V181" s="10">
+        <v>0.58199999999999996</v>
+      </c>
     </row>
     <row r="182" spans="1:22" ht="15.75" customHeight="1">
-      <c r="A182" s="10"/>
-      <c r="B182" s="10"/>
+      <c r="A182" s="13">
+        <v>46307</v>
+      </c>
+      <c r="B182" s="10" t="s">
+        <v>367</v>
+      </c>
       <c r="C182" s="10"/>
       <c r="D182" s="10"/>
       <c r="E182" s="10"/>

</xml_diff>

<commit_message>
numbers chnaged in trust layer
</commit_message>
<xml_diff>
--- a/scratch/tracker.xlsx
+++ b/scratch/tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://drpinnacle-my.sharepoint.com/personal/vish_drpinnacle_com/Documents/Projects/openvals/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3264" documentId="8_{F24D4BFB-FFC1-BD42-9143-22F6B790B9D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B56F1BE5-F1B5-4FDC-9A77-6F61C3D3CFA2}"/>
+  <xr:revisionPtr revIDLastSave="3265" documentId="8_{F24D4BFB-FFC1-BD42-9143-22F6B790B9D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D9AA07F-4022-44CD-B57E-28A384B5C41B}"/>
   <bookViews>
     <workbookView xWindow="3960" yWindow="2780" windowWidth="28040" windowHeight="17180" xr2:uid="{BEF502B7-096A-F24C-A77D-ED0F5F38F7FE}"/>
   </bookViews>
@@ -3264,10 +3264,7 @@
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
-      <c r="L25" s="2">
-        <f>-P12</f>
-        <v>-0.64400000000000002</v>
-      </c>
+      <c r="L25" s="2"/>
       <c r="M25" s="9"/>
       <c r="N25" s="2"/>
       <c r="O25" s="2">

</xml_diff>

<commit_message>
add initial UI components, benchmarks, and layout pages for the openvals website
</commit_message>
<xml_diff>
--- a/scratch/tracker.xlsx
+++ b/scratch/tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://drpinnacle-my.sharepoint.com/personal/vish_drpinnacle_com/Documents/Projects/openvals/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3265" documentId="8_{F24D4BFB-FFC1-BD42-9143-22F6B790B9D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D9AA07F-4022-44CD-B57E-28A384B5C41B}"/>
+  <xr:revisionPtr revIDLastSave="3287" documentId="8_{F24D4BFB-FFC1-BD42-9143-22F6B790B9D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{25FC002F-DB0F-4765-A2E2-ED2AF36C51EC}"/>
   <bookViews>
     <workbookView xWindow="3960" yWindow="2780" windowWidth="28040" windowHeight="17180" xr2:uid="{BEF502B7-096A-F24C-A77D-ED0F5F38F7FE}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1086" uniqueCount="380">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1090" uniqueCount="383">
   <si>
     <t>Date</t>
   </si>
@@ -1182,6 +1182,15 @@
   </si>
   <si>
     <t>935MB</t>
+  </si>
+  <si>
+    <t>falcon-h1</t>
+  </si>
+  <si>
+    <t>448b</t>
+  </si>
+  <si>
+    <t>Tii</t>
   </si>
 </sst>
 </file>
@@ -11407,26 +11416,50 @@
       <c r="B182" s="10" t="s">
         <v>367</v>
       </c>
-      <c r="C182" s="10"/>
-      <c r="D182" s="10"/>
-      <c r="E182" s="10"/>
-      <c r="F182" s="10"/>
+      <c r="C182" t="s">
+        <v>380</v>
+      </c>
+      <c r="D182" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="E182" s="10" t="s">
+        <v>381</v>
+      </c>
+      <c r="F182" s="10" t="s">
+        <v>382</v>
+      </c>
       <c r="G182" s="10"/>
       <c r="H182" s="10"/>
-      <c r="I182" s="10"/>
+      <c r="I182" s="30"/>
       <c r="J182" s="10"/>
       <c r="K182" s="10"/>
       <c r="L182" s="10"/>
       <c r="M182" s="10"/>
       <c r="N182" s="10"/>
-      <c r="O182" s="10"/>
-      <c r="P182" s="10"/>
-      <c r="Q182" s="10"/>
-      <c r="R182" s="10"/>
-      <c r="S182" s="10"/>
-      <c r="T182" s="10"/>
-      <c r="U182" s="10"/>
-      <c r="V182" s="10"/>
+      <c r="O182" s="10">
+        <v>0.83199999999999996</v>
+      </c>
+      <c r="P182" s="10">
+        <v>0.67700000000000005</v>
+      </c>
+      <c r="Q182" s="10">
+        <v>19401.37</v>
+      </c>
+      <c r="R182" s="10">
+        <v>0.73199999999999998</v>
+      </c>
+      <c r="S182" s="10">
+        <v>0.53500000000000003</v>
+      </c>
+      <c r="T182" s="10">
+        <v>0.9</v>
+      </c>
+      <c r="U182" s="10">
+        <v>0.89100000000000001</v>
+      </c>
+      <c r="V182" s="10">
+        <v>0.63600000000000001</v>
+      </c>
     </row>
     <row r="183" spans="1:22" ht="15.75" customHeight="1">
       <c r="A183" s="10"/>

</xml_diff>

<commit_message>
initialize website with layout, branding assets, and benchmark dataset components
</commit_message>
<xml_diff>
--- a/scratch/tracker.xlsx
+++ b/scratch/tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://drpinnacle-my.sharepoint.com/personal/vish_drpinnacle_com/Documents/Projects/openvals/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3306" documentId="8_{F24D4BFB-FFC1-BD42-9143-22F6B790B9D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{22EE77E3-CC00-42F2-86C3-07EB60C8EB60}"/>
+  <xr:revisionPtr revIDLastSave="3344" documentId="8_{F24D4BFB-FFC1-BD42-9143-22F6B790B9D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A7B1043B-F1B2-425C-BC6B-F1495A41E143}"/>
   <bookViews>
     <workbookView xWindow="3960" yWindow="2780" windowWidth="28040" windowHeight="17180" xr2:uid="{BEF502B7-096A-F24C-A77D-ED0F5F38F7FE}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1096" uniqueCount="382">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1110" uniqueCount="390">
   <si>
     <t>Date</t>
   </si>
@@ -1188,6 +1188,30 @@
   </si>
   <si>
     <t>448b</t>
+  </si>
+  <si>
+    <t>exaone-4.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">812 MB </t>
+  </si>
+  <si>
+    <t>LG AI Research</t>
+  </si>
+  <si>
+    <t>ernie-4.5</t>
+  </si>
+  <si>
+    <t>220mb</t>
+  </si>
+  <si>
+    <t>Baidu</t>
+  </si>
+  <si>
+    <t>lfm2-1.2b</t>
+  </si>
+  <si>
+    <t>730mb</t>
   </si>
 </sst>
 </file>
@@ -11517,58 +11541,122 @@
       <c r="B184" s="10" t="s">
         <v>367</v>
       </c>
-      <c r="C184" s="10"/>
-      <c r="D184" s="10"/>
-      <c r="E184" s="10"/>
-      <c r="F184" s="10"/>
+      <c r="C184" t="s">
+        <v>382</v>
+      </c>
+      <c r="D184" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="E184" s="10" t="s">
+        <v>383</v>
+      </c>
+      <c r="F184" t="s">
+        <v>384</v>
+      </c>
       <c r="G184" s="10"/>
       <c r="H184" s="10"/>
       <c r="I184" s="10"/>
       <c r="J184" s="10"/>
-      <c r="K184" s="10"/>
+      <c r="K184" s="30"/>
       <c r="L184" s="10"/>
       <c r="M184" s="10"/>
       <c r="N184" s="10"/>
-      <c r="O184" s="10"/>
-      <c r="P184" s="10"/>
-      <c r="Q184" s="10"/>
-      <c r="R184" s="10"/>
-      <c r="S184" s="10"/>
-      <c r="T184" s="10"/>
-      <c r="U184" s="10"/>
-      <c r="V184" s="10"/>
+      <c r="O184" s="10">
+        <v>0.90200000000000002</v>
+      </c>
+      <c r="P184" s="10">
+        <v>0.41199999999999998</v>
+      </c>
+      <c r="Q184" s="10">
+        <v>48734.2</v>
+      </c>
+      <c r="R184" s="10">
+        <v>0.53</v>
+      </c>
+      <c r="S184" s="10">
+        <v>0.63</v>
+      </c>
+      <c r="T184" s="10">
+        <v>1</v>
+      </c>
+      <c r="U184" s="10">
+        <v>0.86799999999999999</v>
+      </c>
+      <c r="V184" s="10">
+        <v>0.57699999999999996</v>
+      </c>
     </row>
     <row r="185" spans="1:22" ht="15.75" customHeight="1">
-      <c r="A185" s="10"/>
-      <c r="B185" s="10"/>
-      <c r="C185" s="10"/>
-      <c r="D185" s="10"/>
-      <c r="E185" s="10"/>
-      <c r="F185" s="10"/>
+      <c r="A185" s="13">
+        <v>46309</v>
+      </c>
+      <c r="B185" s="10" t="s">
+        <v>367</v>
+      </c>
+      <c r="C185" t="s">
+        <v>385</v>
+      </c>
+      <c r="D185" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="E185" s="10" t="s">
+        <v>386</v>
+      </c>
+      <c r="F185" s="10" t="s">
+        <v>387</v>
+      </c>
       <c r="G185" s="10"/>
       <c r="H185" s="10"/>
       <c r="I185" s="10"/>
       <c r="J185" s="10"/>
-      <c r="K185" s="10"/>
+      <c r="K185" s="30"/>
       <c r="L185" s="10"/>
       <c r="M185" s="10"/>
       <c r="N185" s="10"/>
-      <c r="O185" s="10"/>
-      <c r="P185" s="10"/>
-      <c r="Q185" s="10"/>
-      <c r="R185" s="10"/>
-      <c r="S185" s="10"/>
-      <c r="T185" s="10"/>
-      <c r="U185" s="10"/>
-      <c r="V185" s="10"/>
+      <c r="O185" s="10">
+        <v>0.82</v>
+      </c>
+      <c r="P185" s="10">
+        <v>0.20699999999999999</v>
+      </c>
+      <c r="Q185" s="10">
+        <v>3049.23</v>
+      </c>
+      <c r="R185" s="10">
+        <v>0.36599999999999999</v>
+      </c>
+      <c r="S185" s="10">
+        <v>0.69799999999999995</v>
+      </c>
+      <c r="T185" s="10">
+        <v>1</v>
+      </c>
+      <c r="U185" s="10">
+        <v>0.61199999999999999</v>
+      </c>
+      <c r="V185" s="10">
+        <v>0.32700000000000001</v>
+      </c>
     </row>
     <row r="186" spans="1:22" ht="15.75" customHeight="1">
-      <c r="A186" s="10"/>
-      <c r="B186" s="10"/>
-      <c r="C186" s="10"/>
-      <c r="D186" s="10"/>
-      <c r="E186" s="10"/>
-      <c r="F186" s="10"/>
+      <c r="A186" s="13">
+        <v>46309</v>
+      </c>
+      <c r="B186" s="10" t="s">
+        <v>367</v>
+      </c>
+      <c r="C186" t="s">
+        <v>388</v>
+      </c>
+      <c r="D186" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="E186" s="10" t="s">
+        <v>389</v>
+      </c>
+      <c r="F186" s="10" t="s">
+        <v>79</v>
+      </c>
       <c r="G186" s="10"/>
       <c r="H186" s="10"/>
       <c r="I186" s="10"/>

</xml_diff>

<commit_message>
signup link added in pricing page
</commit_message>
<xml_diff>
--- a/scratch/tracker.xlsx
+++ b/scratch/tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://drpinnacle-my.sharepoint.com/personal/vish_drpinnacle_com/Documents/Projects/openvals/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3443" documentId="8_{F24D4BFB-FFC1-BD42-9143-22F6B790B9D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{050E558B-6D54-4ED9-BB3B-359CC22D3728}"/>
+  <xr:revisionPtr revIDLastSave="3468" documentId="8_{F24D4BFB-FFC1-BD42-9143-22F6B790B9D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{931C1623-46F7-4D57-A494-2980F62ED4A7}"/>
   <bookViews>
     <workbookView xWindow="3960" yWindow="2780" windowWidth="28040" windowHeight="17180" xr2:uid="{BEF502B7-096A-F24C-A77D-ED0F5F38F7FE}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1133" uniqueCount="408">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1143" uniqueCount="413">
   <si>
     <t>Date</t>
   </si>
@@ -1266,6 +1266,21 @@
   </si>
   <si>
     <t>4,230.32 ms</t>
+  </si>
+  <si>
+    <t>gemma3:1b</t>
+  </si>
+  <si>
+    <t>1B</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 883 MB </t>
+  </si>
+  <si>
+    <t>hunyuan-0.5b-instruct</t>
+  </si>
+  <si>
+    <t>320mb</t>
   </si>
 </sst>
 </file>
@@ -11953,12 +11968,24 @@
       </c>
     </row>
     <row r="191" spans="1:22" ht="15.75" customHeight="1">
-      <c r="A191" s="10"/>
-      <c r="B191" s="10"/>
-      <c r="C191" s="10"/>
-      <c r="D191" s="10"/>
-      <c r="E191" s="10"/>
-      <c r="F191" s="10"/>
+      <c r="A191" s="13">
+        <v>46309</v>
+      </c>
+      <c r="B191" s="10" t="s">
+        <v>393</v>
+      </c>
+      <c r="C191" t="s">
+        <v>408</v>
+      </c>
+      <c r="D191" t="s">
+        <v>409</v>
+      </c>
+      <c r="E191" s="10" t="s">
+        <v>410</v>
+      </c>
+      <c r="F191" t="s">
+        <v>74</v>
+      </c>
       <c r="G191" s="10"/>
       <c r="H191" s="10"/>
       <c r="I191" s="10"/>
@@ -11977,28 +12004,56 @@
       <c r="V191" s="10"/>
     </row>
     <row r="192" spans="1:22" ht="15.75" customHeight="1">
-      <c r="A192" s="10"/>
-      <c r="B192" s="10"/>
-      <c r="C192" s="10"/>
-      <c r="D192" s="10"/>
-      <c r="E192" s="10"/>
-      <c r="F192" s="10"/>
+      <c r="A192" s="13">
+        <v>46309</v>
+      </c>
+      <c r="B192" s="10" t="s">
+        <v>367</v>
+      </c>
+      <c r="C192" t="s">
+        <v>411</v>
+      </c>
+      <c r="D192" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="E192" s="10" t="s">
+        <v>412</v>
+      </c>
+      <c r="F192" s="10" t="s">
+        <v>208</v>
+      </c>
       <c r="G192" s="10"/>
       <c r="H192" s="10"/>
       <c r="I192" s="10"/>
       <c r="J192" s="10"/>
-      <c r="K192" s="10"/>
+      <c r="K192" s="30"/>
       <c r="L192" s="10"/>
       <c r="M192" s="10"/>
       <c r="N192" s="10"/>
-      <c r="O192" s="10"/>
-      <c r="P192" s="10"/>
-      <c r="Q192" s="10"/>
-      <c r="R192" s="10"/>
-      <c r="S192" s="10"/>
-      <c r="T192" s="10"/>
-      <c r="U192" s="10"/>
-      <c r="V192" s="10"/>
+      <c r="O192" s="10">
+        <v>0.85199999999999998</v>
+      </c>
+      <c r="P192" s="10">
+        <v>0.38300000000000001</v>
+      </c>
+      <c r="Q192" s="10">
+        <v>29509.200000000001</v>
+      </c>
+      <c r="R192" s="10">
+        <v>0.50600000000000001</v>
+      </c>
+      <c r="S192" s="10">
+        <v>0.63600000000000001</v>
+      </c>
+      <c r="T192" s="10">
+        <v>1</v>
+      </c>
+      <c r="U192" s="10">
+        <v>0.76300000000000001</v>
+      </c>
+      <c r="V192" s="10">
+        <v>0.54300000000000004</v>
+      </c>
     </row>
     <row r="193" spans="1:22" ht="15.75" customHeight="1">
       <c r="A193" s="10"/>

</xml_diff>

<commit_message>
alignment fix in landing page
</commit_message>
<xml_diff>
--- a/scratch/tracker.xlsx
+++ b/scratch/tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://drpinnacle-my.sharepoint.com/personal/vish_drpinnacle_com/Documents/Projects/openvals/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3470" documentId="8_{F24D4BFB-FFC1-BD42-9143-22F6B790B9D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{361B1619-D51C-4D88-AE4C-082256B67C2B}"/>
+  <xr:revisionPtr revIDLastSave="3485" documentId="8_{F24D4BFB-FFC1-BD42-9143-22F6B790B9D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{01BFD835-7A02-4109-AE4E-9FCAB74BD136}"/>
   <bookViews>
     <workbookView xWindow="3960" yWindow="2780" windowWidth="28040" windowHeight="17180" xr2:uid="{BEF502B7-096A-F24C-A77D-ED0F5F38F7FE}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1144" uniqueCount="414">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1149" uniqueCount="416">
   <si>
     <t>Date</t>
   </si>
@@ -1284,6 +1284,12 @@
   </si>
   <si>
     <t>320mb</t>
+  </si>
+  <si>
+    <t>llama3.2:1b-instruct-q5_K_M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">800MB </t>
   </si>
 </sst>
 </file>
@@ -2166,7 +2172,7 @@
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="2" max="2" width="10.375" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="3" max="3" width="26.75" customWidth="1"/>
     <col min="6" max="6" width="13.25" customWidth="1"/>
     <col min="8" max="8" width="14.625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.625" bestFit="1" customWidth="1"/>
@@ -12075,12 +12081,22 @@
       </c>
     </row>
     <row r="193" spans="1:22" ht="15.75" customHeight="1">
-      <c r="A193" s="10"/>
-      <c r="B193" s="10"/>
-      <c r="C193" s="10"/>
+      <c r="A193" s="13">
+        <v>46310</v>
+      </c>
+      <c r="B193" s="10" t="s">
+        <v>393</v>
+      </c>
+      <c r="C193" t="s">
+        <v>414</v>
+      </c>
       <c r="D193" s="10"/>
-      <c r="E193" s="10"/>
-      <c r="F193" s="10"/>
+      <c r="E193" s="10" t="s">
+        <v>415</v>
+      </c>
+      <c r="F193" t="s">
+        <v>43</v>
+      </c>
       <c r="G193" s="10"/>
       <c r="H193" s="10"/>
       <c r="I193" s="10"/>
@@ -12088,20 +12104,35 @@
       <c r="K193" s="10"/>
       <c r="L193" s="10"/>
       <c r="M193" s="10"/>
-      <c r="N193" s="10"/>
-      <c r="O193" s="10"/>
-      <c r="P193" s="10"/>
-      <c r="Q193" s="10"/>
-      <c r="R193" s="10"/>
-      <c r="S193" s="10"/>
-      <c r="T193" s="10"/>
-      <c r="U193" s="10"/>
-      <c r="V193" s="10"/>
+      <c r="N193" s="30"/>
+      <c r="O193">
+        <v>0.66100000000000003</v>
+      </c>
+      <c r="P193">
+        <v>0.63100000000000001</v>
+      </c>
+      <c r="Q193" t="s">
+        <v>411</v>
+      </c>
+      <c r="R193">
+        <v>0.70499999999999996</v>
+      </c>
+      <c r="S193">
+        <v>0.55500000000000005</v>
+      </c>
+      <c r="T193">
+        <v>0.97</v>
+      </c>
+      <c r="U193">
+        <v>0.81599999999999995</v>
+      </c>
+      <c r="V193">
+        <v>0.57799999999999996</v>
+      </c>
     </row>
     <row r="194" spans="1:22" ht="15.75" customHeight="1">
-      <c r="A194" s="10"/>
+      <c r="A194" s="13"/>
       <c r="B194" s="10"/>
-      <c r="C194" s="10"/>
       <c r="D194" s="10"/>
       <c r="E194" s="10"/>
       <c r="F194" s="10"/>

</xml_diff>

<commit_message>
add OpenVals website components, pages, and benchmark datasets
</commit_message>
<xml_diff>
--- a/scratch/tracker.xlsx
+++ b/scratch/tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://drpinnacle-my.sharepoint.com/personal/vish_drpinnacle_com/Documents/Projects/openvals/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3697" documentId="8_{F24D4BFB-FFC1-BD42-9143-22F6B790B9D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{27518C61-5283-4F14-ACDC-9826A2D50C43}"/>
+  <xr:revisionPtr revIDLastSave="3964" documentId="8_{F24D4BFB-FFC1-BD42-9143-22F6B790B9D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE32F0F1-F4BF-48BD-8129-3D1AE406121E}"/>
   <bookViews>
     <workbookView xWindow="3960" yWindow="2780" windowWidth="28040" windowHeight="17180" xr2:uid="{BEF502B7-096A-F24C-A77D-ED0F5F38F7FE}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1240" uniqueCount="476">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1329" uniqueCount="522">
   <si>
     <t>Date</t>
   </si>
@@ -1470,6 +1470,144 @@
   </si>
   <si>
     <t>678.99 ms</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> gemma4:e2b</t>
+  </si>
+  <si>
+    <t>2B</t>
+  </si>
+  <si>
+    <t>~4.6 GB</t>
+  </si>
+  <si>
+    <t>5721.52 ms</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> deepcoder:1.5b</t>
+  </si>
+  <si>
+    <t>1.5B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.1 GB </t>
+  </si>
+  <si>
+    <t>smollm:1.7b-instruct-v0.2-q4_K_M</t>
+  </si>
+  <si>
+    <t>1.7B</t>
+  </si>
+  <si>
+    <t>Qwen2 1.5B</t>
+  </si>
+  <si>
+    <t>934 MB</t>
+  </si>
+  <si>
+    <t>Medllama-1B-Instruct-v3-GGUF:Q4_K_M</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 807 MB</t>
+  </si>
+  <si>
+    <t>Llama SmolTalk 3.2 1B Instruct Q4_K_M</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 672 MB</t>
+  </si>
+  <si>
+    <t>KittyLM MiniCPM5 1B</t>
+  </si>
+  <si>
+    <t>377.33 ms</t>
+  </si>
+  <si>
+    <t>atlas-coder</t>
+  </si>
+  <si>
+    <t>531 Mb</t>
+  </si>
+  <si>
+    <t>Pluto AI Labs</t>
+  </si>
+  <si>
+    <t>157380.2MS</t>
+  </si>
+  <si>
+    <t>LFM2.5-1.2B Thinking</t>
+  </si>
+  <si>
+    <t>731mb</t>
+  </si>
+  <si>
+    <t>Falcon3:1b</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1.8 GB</t>
+  </si>
+  <si>
+    <t>1369.01 ms</t>
+  </si>
+  <si>
+    <t>StableLM Zephyr 1.6B</t>
+  </si>
+  <si>
+    <t>1.6B</t>
+  </si>
+  <si>
+    <t>980MB</t>
+  </si>
+  <si>
+    <t>741.99 ms</t>
+  </si>
+  <si>
+    <t>orca-mini:3b</t>
+  </si>
+  <si>
+    <t>355.08 ms</t>
+  </si>
+  <si>
+    <t>stable-beluga:latest</t>
+  </si>
+  <si>
+    <t>1138.41 ms</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> qwen2:1.5b</t>
+  </si>
+  <si>
+    <t>597.96 ms</t>
+  </si>
+  <si>
+    <t>openelm</t>
+  </si>
+  <si>
+    <t>0.45b</t>
+  </si>
+  <si>
+    <t>289 MB</t>
+  </si>
+  <si>
+    <t>Apple</t>
+  </si>
+  <si>
+    <t>11827.33 ms</t>
+  </si>
+  <si>
+    <t>pythia</t>
+  </si>
+  <si>
+    <t>0.41b</t>
+  </si>
+  <si>
+    <t>267mb</t>
+  </si>
+  <si>
+    <t>EleutherAI</t>
+  </si>
+  <si>
+    <t>9333.3ms</t>
   </si>
 </sst>
 </file>
@@ -2383,7 +2521,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A897CD1C-0E15-574E-9F3A-4CBFEDFF084C}">
-  <dimension ref="A1:V208"/>
+  <dimension ref="A1:V224"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="2" max="2" width="10.375" customWidth="1"/>
@@ -13124,6 +13262,829 @@
         <v>0.57299999999999995</v>
       </c>
     </row>
+    <row r="209" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A209" s="13">
+        <v>46321</v>
+      </c>
+      <c r="B209" s="10" t="s">
+        <v>393</v>
+      </c>
+      <c r="C209" t="s">
+        <v>476</v>
+      </c>
+      <c r="D209" t="s">
+        <v>477</v>
+      </c>
+      <c r="E209" t="s">
+        <v>478</v>
+      </c>
+      <c r="F209" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="G209" s="2"/>
+      <c r="H209" s="2"/>
+      <c r="I209" s="2"/>
+      <c r="J209" s="2"/>
+      <c r="K209" s="30"/>
+      <c r="L209" s="2"/>
+      <c r="M209" s="2"/>
+      <c r="N209" s="2"/>
+      <c r="O209">
+        <v>0.72299999999999998</v>
+      </c>
+      <c r="P209">
+        <v>0.501</v>
+      </c>
+      <c r="Q209" t="s">
+        <v>479</v>
+      </c>
+      <c r="R209">
+        <v>0.60099999999999998</v>
+      </c>
+      <c r="S209">
+        <v>1</v>
+      </c>
+      <c r="T209">
+        <v>0.71499999999999997</v>
+      </c>
+      <c r="U209">
+        <v>1</v>
+      </c>
+      <c r="V209">
+        <v>0.53400000000000003</v>
+      </c>
+    </row>
+    <row r="210" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A210" s="13">
+        <v>46321</v>
+      </c>
+      <c r="B210" s="10" t="s">
+        <v>393</v>
+      </c>
+      <c r="C210" t="s">
+        <v>480</v>
+      </c>
+      <c r="D210" t="s">
+        <v>481</v>
+      </c>
+      <c r="E210" s="2" t="s">
+        <v>482</v>
+      </c>
+      <c r="F210" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="G210" s="2"/>
+      <c r="H210" s="2"/>
+      <c r="I210" s="2"/>
+      <c r="J210" s="2"/>
+      <c r="K210" s="30"/>
+      <c r="L210" s="2"/>
+      <c r="M210" s="2"/>
+      <c r="N210" s="2"/>
+      <c r="O210">
+        <v>0.307</v>
+      </c>
+      <c r="P210">
+        <v>0.34799999999999998</v>
+      </c>
+      <c r="Q210">
+        <v>227.69</v>
+      </c>
+      <c r="R210">
+        <v>0.47899999999999998</v>
+      </c>
+      <c r="S210">
+        <v>0.63400000000000001</v>
+      </c>
+      <c r="T210">
+        <v>1</v>
+      </c>
+      <c r="U210">
+        <v>0.38700000000000001</v>
+      </c>
+      <c r="V210">
+        <v>0.39600000000000002</v>
+      </c>
+    </row>
+    <row r="211" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A211" s="13">
+        <v>46321</v>
+      </c>
+      <c r="B211" s="10" t="s">
+        <v>393</v>
+      </c>
+      <c r="C211" t="s">
+        <v>483</v>
+      </c>
+      <c r="D211" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="E211" s="2" t="s">
+        <v>482</v>
+      </c>
+      <c r="F211" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="G211" s="2"/>
+      <c r="H211" s="2"/>
+      <c r="I211" s="2"/>
+      <c r="J211" s="2"/>
+      <c r="K211" s="30"/>
+      <c r="L211" s="2"/>
+      <c r="M211" s="2"/>
+      <c r="N211" s="2"/>
+      <c r="O211">
+        <v>0.71799999999999997</v>
+      </c>
+      <c r="P211">
+        <v>0.439</v>
+      </c>
+      <c r="Q211">
+        <v>1771.27</v>
+      </c>
+      <c r="R211">
+        <v>0.55100000000000005</v>
+      </c>
+      <c r="S211">
+        <v>0.61699999999999999</v>
+      </c>
+      <c r="T211">
+        <v>0.90500000000000003</v>
+      </c>
+      <c r="U211">
+        <v>0.92100000000000004</v>
+      </c>
+      <c r="V211">
+        <v>0.55200000000000005</v>
+      </c>
+    </row>
+    <row r="212" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A212" s="13">
+        <v>46321</v>
+      </c>
+      <c r="B212" s="10" t="s">
+        <v>398</v>
+      </c>
+      <c r="C212" t="s">
+        <v>485</v>
+      </c>
+      <c r="D212" t="s">
+        <v>481</v>
+      </c>
+      <c r="E212" s="2" t="s">
+        <v>486</v>
+      </c>
+      <c r="F212" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="G212" s="2"/>
+      <c r="H212" s="2"/>
+      <c r="I212" s="2"/>
+      <c r="J212" s="2"/>
+      <c r="K212" s="30"/>
+      <c r="L212" s="2"/>
+      <c r="M212" s="2"/>
+      <c r="N212" s="2"/>
+      <c r="O212">
+        <v>0.76800000000000002</v>
+      </c>
+      <c r="P212">
+        <v>0.54200000000000004</v>
+      </c>
+      <c r="Q212">
+        <v>795.2</v>
+      </c>
+      <c r="R212">
+        <v>0.63400000000000001</v>
+      </c>
+      <c r="S212">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="T212">
+        <v>0.90500000000000003</v>
+      </c>
+      <c r="U212">
+        <v>0.85199999999999998</v>
+      </c>
+      <c r="V212">
+        <v>0.59099999999999997</v>
+      </c>
+    </row>
+    <row r="213" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A213" s="13">
+        <v>46321</v>
+      </c>
+      <c r="B213" s="10" t="s">
+        <v>398</v>
+      </c>
+      <c r="C213" s="12" t="s">
+        <v>487</v>
+      </c>
+      <c r="D213" s="2"/>
+      <c r="E213" s="2" t="s">
+        <v>488</v>
+      </c>
+      <c r="F213" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="G213" s="2"/>
+      <c r="H213" s="2"/>
+      <c r="I213" s="2"/>
+      <c r="J213" s="2"/>
+      <c r="K213" s="30"/>
+      <c r="L213" s="2"/>
+      <c r="M213" s="2"/>
+      <c r="N213" s="2"/>
+      <c r="O213">
+        <v>0.754</v>
+      </c>
+      <c r="P213">
+        <v>0.45200000000000001</v>
+      </c>
+      <c r="Q213">
+        <v>1069.24</v>
+      </c>
+      <c r="R213">
+        <v>0.56200000000000006</v>
+      </c>
+      <c r="S213">
+        <v>0.61199999999999999</v>
+      </c>
+      <c r="T213">
+        <v>1</v>
+      </c>
+      <c r="U213">
+        <v>0.88800000000000001</v>
+      </c>
+      <c r="V213">
+        <v>0.57599999999999996</v>
+      </c>
+    </row>
+    <row r="214" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A214" s="13">
+        <v>46321</v>
+      </c>
+      <c r="B214" s="10" t="s">
+        <v>393</v>
+      </c>
+      <c r="C214" s="12" t="s">
+        <v>489</v>
+      </c>
+      <c r="D214" t="s">
+        <v>409</v>
+      </c>
+      <c r="E214" s="2" t="s">
+        <v>490</v>
+      </c>
+      <c r="F214" t="s">
+        <v>69</v>
+      </c>
+      <c r="G214" s="2"/>
+      <c r="H214" s="2"/>
+      <c r="I214" s="2"/>
+      <c r="J214" s="2"/>
+      <c r="K214" s="30"/>
+      <c r="L214" s="2"/>
+      <c r="M214" s="2"/>
+      <c r="N214" s="2"/>
+      <c r="O214">
+        <v>0.81599999999999995</v>
+      </c>
+      <c r="P214">
+        <v>0.44600000000000001</v>
+      </c>
+      <c r="Q214">
+        <v>1279.92</v>
+      </c>
+      <c r="R214">
+        <v>0.55700000000000005</v>
+      </c>
+      <c r="S214">
+        <v>0.61399999999999999</v>
+      </c>
+      <c r="T214">
+        <v>1</v>
+      </c>
+      <c r="U214">
+        <v>0.83799999999999997</v>
+      </c>
+      <c r="V214">
+        <v>0.57699999999999996</v>
+      </c>
+    </row>
+    <row r="215" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A215" s="13">
+        <v>46321</v>
+      </c>
+      <c r="B215" s="10" t="s">
+        <v>398</v>
+      </c>
+      <c r="C215" t="s">
+        <v>491</v>
+      </c>
+      <c r="D215" t="s">
+        <v>409</v>
+      </c>
+      <c r="E215" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="F215" t="s">
+        <v>69</v>
+      </c>
+      <c r="G215" s="2"/>
+      <c r="H215" s="2"/>
+      <c r="I215" s="2"/>
+      <c r="J215" s="2"/>
+      <c r="K215" s="30"/>
+      <c r="L215" s="2"/>
+      <c r="M215" s="2"/>
+      <c r="N215" s="2"/>
+      <c r="O215">
+        <v>0.14799999999999999</v>
+      </c>
+      <c r="P215">
+        <v>0.37</v>
+      </c>
+      <c r="Q215" t="s">
+        <v>492</v>
+      </c>
+      <c r="R215">
+        <v>0.496</v>
+      </c>
+      <c r="S215">
+        <v>0.63700000000000001</v>
+      </c>
+      <c r="T215">
+        <v>1</v>
+      </c>
+      <c r="U215">
+        <v>0.63</v>
+      </c>
+      <c r="V215">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="216" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A216" s="13">
+        <v>46321</v>
+      </c>
+      <c r="B216" s="10" t="s">
+        <v>367</v>
+      </c>
+      <c r="C216" t="s">
+        <v>493</v>
+      </c>
+      <c r="D216" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="E216" s="2" t="s">
+        <v>494</v>
+      </c>
+      <c r="F216" t="s">
+        <v>495</v>
+      </c>
+      <c r="G216" s="23"/>
+      <c r="H216" s="2"/>
+      <c r="I216" s="2"/>
+      <c r="J216" s="2"/>
+      <c r="K216" s="2"/>
+      <c r="L216" s="2"/>
+      <c r="M216" s="2"/>
+      <c r="N216" s="2"/>
+      <c r="O216" s="2">
+        <v>0.51200000000000001</v>
+      </c>
+      <c r="P216" s="2">
+        <v>0.40400000000000003</v>
+      </c>
+      <c r="Q216" s="2" t="s">
+        <v>496</v>
+      </c>
+      <c r="R216" s="2">
+        <v>0.52300000000000002</v>
+      </c>
+      <c r="S216" s="2">
+        <v>0.63700000000000001</v>
+      </c>
+      <c r="T216" s="2">
+        <v>0.97</v>
+      </c>
+      <c r="U216" s="4">
+        <v>0.77800000000000002</v>
+      </c>
+      <c r="V216" s="6">
+        <v>0.48</v>
+      </c>
+    </row>
+    <row r="217" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A217" s="13">
+        <v>46321</v>
+      </c>
+      <c r="B217" s="10" t="s">
+        <v>393</v>
+      </c>
+      <c r="C217" t="s">
+        <v>497</v>
+      </c>
+      <c r="D217" s="2" t="s">
+        <v>477</v>
+      </c>
+      <c r="E217" s="2" t="s">
+        <v>498</v>
+      </c>
+      <c r="F217" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="G217" s="23"/>
+      <c r="H217" s="2"/>
+      <c r="I217" s="2"/>
+      <c r="J217" s="2"/>
+      <c r="K217" s="2"/>
+      <c r="L217" s="2"/>
+      <c r="M217" s="2"/>
+      <c r="N217" s="2"/>
+      <c r="O217">
+        <v>0.75900000000000001</v>
+      </c>
+      <c r="P217">
+        <v>0.63700000000000001</v>
+      </c>
+      <c r="Q217">
+        <v>0.71</v>
+      </c>
+      <c r="R217">
+        <v>0.90600000000000003</v>
+      </c>
+      <c r="S217">
+        <v>1</v>
+      </c>
+      <c r="T217">
+        <v>0.33300000000000002</v>
+      </c>
+      <c r="U217">
+        <v>1</v>
+      </c>
+      <c r="V217">
+        <v>0.54700000000000004</v>
+      </c>
+    </row>
+    <row r="218" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A218" s="13">
+        <v>46321</v>
+      </c>
+      <c r="B218" s="10" t="s">
+        <v>398</v>
+      </c>
+      <c r="C218" t="s">
+        <v>499</v>
+      </c>
+      <c r="D218" t="s">
+        <v>409</v>
+      </c>
+      <c r="E218" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="F218" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="G218" s="23"/>
+      <c r="H218" s="2"/>
+      <c r="I218" s="2"/>
+      <c r="J218" s="2"/>
+      <c r="K218" s="2"/>
+      <c r="L218" s="2"/>
+      <c r="M218" s="2"/>
+      <c r="N218" s="2"/>
+      <c r="O218">
+        <v>0.78800000000000003</v>
+      </c>
+      <c r="P218">
+        <v>0.624</v>
+      </c>
+      <c r="Q218" t="s">
+        <v>501</v>
+      </c>
+      <c r="R218">
+        <v>0.69899999999999995</v>
+      </c>
+      <c r="S218">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="T218">
+        <v>1</v>
+      </c>
+      <c r="U218">
+        <v>0.81499999999999995</v>
+      </c>
+      <c r="V218">
+        <v>0.61799999999999999</v>
+      </c>
+    </row>
+    <row r="219" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A219" s="13">
+        <v>46321</v>
+      </c>
+      <c r="B219" s="10" t="s">
+        <v>393</v>
+      </c>
+      <c r="C219" t="s">
+        <v>502</v>
+      </c>
+      <c r="D219" s="2" t="s">
+        <v>503</v>
+      </c>
+      <c r="E219" s="2" t="s">
+        <v>504</v>
+      </c>
+      <c r="F219" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="G219" s="2"/>
+      <c r="H219" s="2"/>
+      <c r="I219" s="2"/>
+      <c r="J219" s="2"/>
+      <c r="K219" s="2"/>
+      <c r="L219" s="2"/>
+      <c r="M219" s="2"/>
+      <c r="N219" s="30"/>
+      <c r="O219">
+        <v>0.66700000000000004</v>
+      </c>
+      <c r="P219">
+        <v>0.624</v>
+      </c>
+      <c r="Q219" t="s">
+        <v>505</v>
+      </c>
+      <c r="R219">
+        <v>0.69899999999999995</v>
+      </c>
+      <c r="S219">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="T219">
+        <v>1</v>
+      </c>
+      <c r="U219">
+        <v>0.85299999999999998</v>
+      </c>
+      <c r="V219">
+        <v>0.60399999999999998</v>
+      </c>
+    </row>
+    <row r="220" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A220" s="13">
+        <v>46321</v>
+      </c>
+      <c r="B220" s="10" t="s">
+        <v>398</v>
+      </c>
+      <c r="C220" s="12" t="s">
+        <v>506</v>
+      </c>
+      <c r="D220" t="s">
+        <v>468</v>
+      </c>
+      <c r="E220" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F220" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="G220" s="2"/>
+      <c r="H220" s="2"/>
+      <c r="I220" s="2"/>
+      <c r="J220" s="2"/>
+      <c r="K220" s="30"/>
+      <c r="L220" s="2"/>
+      <c r="M220" s="2"/>
+      <c r="N220" s="2"/>
+      <c r="O220">
+        <v>0.63200000000000001</v>
+      </c>
+      <c r="P220">
+        <v>0.48799999999999999</v>
+      </c>
+      <c r="Q220" t="s">
+        <v>507</v>
+      </c>
+      <c r="R220">
+        <v>0.59099999999999997</v>
+      </c>
+      <c r="S220">
+        <v>0.59599999999999997</v>
+      </c>
+      <c r="T220" s="2">
+        <v>1</v>
+      </c>
+      <c r="U220">
+        <v>0.84599999999999997</v>
+      </c>
+      <c r="V220">
+        <v>0.56299999999999994</v>
+      </c>
+    </row>
+    <row r="221" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A221" s="13">
+        <v>46321</v>
+      </c>
+      <c r="B221" s="10" t="s">
+        <v>393</v>
+      </c>
+      <c r="C221" t="s">
+        <v>508</v>
+      </c>
+      <c r="D221" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="E221" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="F221" t="s">
+        <v>88</v>
+      </c>
+      <c r="G221" s="2"/>
+      <c r="H221" s="2"/>
+      <c r="I221" s="2"/>
+      <c r="J221" s="2"/>
+      <c r="K221" s="2"/>
+      <c r="L221" s="2"/>
+      <c r="M221" s="2"/>
+      <c r="N221" s="30"/>
+      <c r="O221">
+        <v>0.55500000000000005</v>
+      </c>
+      <c r="P221">
+        <v>0.53</v>
+      </c>
+      <c r="Q221" t="s">
+        <v>509</v>
+      </c>
+      <c r="R221">
+        <v>0.624</v>
+      </c>
+      <c r="S221">
+        <v>0.58099999999999996</v>
+      </c>
+      <c r="T221">
+        <v>1</v>
+      </c>
+      <c r="U221">
+        <v>0.90100000000000002</v>
+      </c>
+      <c r="V221">
+        <v>0.55900000000000005</v>
+      </c>
+    </row>
+    <row r="222" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A222" s="13">
+        <v>46321</v>
+      </c>
+      <c r="B222" s="10" t="s">
+        <v>398</v>
+      </c>
+      <c r="C222" t="s">
+        <v>510</v>
+      </c>
+      <c r="D222" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E222" s="2" t="s">
+        <v>486</v>
+      </c>
+      <c r="F222" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="G222" s="2"/>
+      <c r="H222" s="2"/>
+      <c r="I222" s="2"/>
+      <c r="J222" s="2"/>
+      <c r="K222" s="2"/>
+      <c r="L222" s="2"/>
+      <c r="M222" s="2"/>
+      <c r="N222" s="30"/>
+      <c r="O222">
+        <v>0.78900000000000003</v>
+      </c>
+      <c r="P222">
+        <v>0.60099999999999998</v>
+      </c>
+      <c r="Q222" t="s">
+        <v>511</v>
+      </c>
+      <c r="R222">
+        <v>0.68100000000000005</v>
+      </c>
+      <c r="S222">
+        <v>0.55600000000000005</v>
+      </c>
+      <c r="T222">
+        <v>1</v>
+      </c>
+      <c r="U222">
+        <v>0.80200000000000005</v>
+      </c>
+      <c r="V222">
+        <v>0.61599999999999999</v>
+      </c>
+    </row>
+    <row r="223" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A223" s="13">
+        <v>46321</v>
+      </c>
+      <c r="B223" s="10" t="s">
+        <v>367</v>
+      </c>
+      <c r="C223" t="s">
+        <v>512</v>
+      </c>
+      <c r="D223" t="s">
+        <v>513</v>
+      </c>
+      <c r="E223" t="s">
+        <v>514</v>
+      </c>
+      <c r="F223" s="2" t="s">
+        <v>515</v>
+      </c>
+      <c r="G223" s="23"/>
+      <c r="H223" s="2"/>
+      <c r="I223" s="2"/>
+      <c r="J223" s="2"/>
+      <c r="K223" s="2"/>
+      <c r="L223" s="2"/>
+      <c r="M223" s="2"/>
+      <c r="N223" s="2"/>
+      <c r="O223">
+        <v>0.22900000000000001</v>
+      </c>
+      <c r="P223">
+        <v>0.34300000000000003</v>
+      </c>
+      <c r="Q223" t="s">
+        <v>516</v>
+      </c>
+      <c r="R223">
+        <v>0.45500000000000002</v>
+      </c>
+      <c r="S223">
+        <v>0.65400000000000003</v>
+      </c>
+      <c r="T223" s="2">
+        <v>1</v>
+      </c>
+      <c r="U223" s="4">
+        <v>0.52</v>
+      </c>
+      <c r="V223" s="6">
+        <v>0.36899999999999999</v>
+      </c>
+    </row>
+    <row r="224" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A224" s="33">
+        <v>46321</v>
+      </c>
+      <c r="B224" t="s">
+        <v>367</v>
+      </c>
+      <c r="C224" t="s">
+        <v>517</v>
+      </c>
+      <c r="D224" t="s">
+        <v>518</v>
+      </c>
+      <c r="E224" t="s">
+        <v>519</v>
+      </c>
+      <c r="F224" t="s">
+        <v>520</v>
+      </c>
+      <c r="G224" s="23"/>
+      <c r="O224">
+        <v>0.217</v>
+      </c>
+      <c r="P224">
+        <v>0.23300000000000001</v>
+      </c>
+      <c r="Q224" t="s">
+        <v>521</v>
+      </c>
+      <c r="R224">
+        <v>0.33800000000000002</v>
+      </c>
+      <c r="S224">
+        <v>0.69</v>
+      </c>
+      <c r="T224">
+        <v>1</v>
+      </c>
+      <c r="U224">
+        <v>0.32500000000000001</v>
+      </c>
+      <c r="V224">
+        <v>0.30199999999999999</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A2:A4"/>

</xml_diff>

<commit_message>
scaffold initial website layout, documentation, and model benchmarking data components
</commit_message>
<xml_diff>
--- a/scratch/tracker.xlsx
+++ b/scratch/tracker.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30621"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://drpinnacle-my.sharepoint.com/personal/vish_drpinnacle_com/Documents/Projects/openvals/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3964" documentId="8_{F24D4BFB-FFC1-BD42-9143-22F6B790B9D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE32F0F1-F4BF-48BD-8129-3D1AE406121E}"/>
+  <xr:revisionPtr revIDLastSave="4244" documentId="8_{F24D4BFB-FFC1-BD42-9143-22F6B790B9D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C43EDE8A-B74A-4D47-BC10-02FE8F00520B}"/>
   <bookViews>
     <workbookView xWindow="3960" yWindow="2780" windowWidth="28040" windowHeight="17180" xr2:uid="{BEF502B7-096A-F24C-A77D-ED0F5F38F7FE}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1329" uniqueCount="522">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1438" uniqueCount="581">
   <si>
     <t>Date</t>
   </si>
@@ -1508,6 +1508,9 @@
     <t>Medllama-1B-Instruct-v3-GGUF:Q4_K_M</t>
   </si>
   <si>
+    <t>1 B</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 807 MB</t>
   </si>
   <si>
@@ -1608,13 +1611,199 @@
   </si>
   <si>
     <t>9333.3ms</t>
+  </si>
+  <si>
+    <t>Llama 3.2 1B Instruct (Q4_K_M)</t>
+  </si>
+  <si>
+    <t>807mb</t>
+  </si>
+  <si>
+    <t>765.95 ms</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> neural-chat:7b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    4.7 GB</t>
+  </si>
+  <si>
+    <t>1356.38 ms</t>
+  </si>
+  <si>
+    <t>dolphin-phi</t>
+  </si>
+  <si>
+    <t>1.6GB</t>
+  </si>
+  <si>
+    <t>954.49 ms</t>
+  </si>
+  <si>
+    <t>dolphin-mistral:latest</t>
+  </si>
+  <si>
+    <t>1548.55 ms</t>
+  </si>
+  <si>
+    <t>granite3.1-dense:2b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.6GB </t>
+  </si>
+  <si>
+    <t>1503.92 ms</t>
+  </si>
+  <si>
+    <t>openhermes:latest</t>
+  </si>
+  <si>
+    <t>Teknium</t>
+  </si>
+  <si>
+    <t>1460.91 ms</t>
+  </si>
+  <si>
+    <t>5741.76 ms</t>
+  </si>
+  <si>
+    <t>xwinlm:7b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7b </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 3.8 GB</t>
+  </si>
+  <si>
+    <r>
+      <t>Xwin-LM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> team</t>
+    </r>
+  </si>
+  <si>
+    <t>4550.93 ms</t>
+  </si>
+  <si>
+    <t>starling-lm:7b</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 4.1 GB</t>
+  </si>
+  <si>
+    <t>nexusflow</t>
+  </si>
+  <si>
+    <t>3069.47 ms</t>
+  </si>
+  <si>
+    <t>falcon:7b-instruct</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 4.2 GB</t>
+  </si>
+  <si>
+    <t>Technology Innovation Institute</t>
+  </si>
+  <si>
+    <t>512.88 ms</t>
+  </si>
+  <si>
+    <t>qwen2.5:1.5b</t>
+  </si>
+  <si>
+    <t>Alibaba Cloud (Qwen team)</t>
+  </si>
+  <si>
+    <t>1587.89 ms</t>
+  </si>
+  <si>
+    <t>qwen2.5:3b</t>
+  </si>
+  <si>
+    <t>3b</t>
+  </si>
+  <si>
+    <t>1.9GB</t>
+  </si>
+  <si>
+    <t>1360.21 ms</t>
+  </si>
+  <si>
+    <t>qwen3:1.7b</t>
+  </si>
+  <si>
+    <t>1.4GB</t>
+  </si>
+  <si>
+    <t>6113.64 ms</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> gemma2:2b</t>
+  </si>
+  <si>
+    <t>2.2b</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1.6 GB</t>
+  </si>
+  <si>
+    <t>2703.15 ms</t>
+  </si>
+  <si>
+    <t>sam860/olmo2:1b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Allem Institute </t>
+  </si>
+  <si>
+    <t>1341.61 ms</t>
+  </si>
+  <si>
+    <t>opencoder:1.5b-instruct-q4_K_M</t>
+  </si>
+  <si>
+    <t>Infly</t>
+  </si>
+  <si>
+    <t>1515.96 ms</t>
+  </si>
+  <si>
+    <t>smollm:1.7b</t>
+  </si>
+  <si>
+    <t>1GB</t>
+  </si>
+  <si>
+    <t>1562.33 ms</t>
+  </si>
+  <si>
+    <t>hf.co/dengcao/ERNIE-4.5-0.3B-PT-GGUF:Q4_K_M</t>
+  </si>
+  <si>
+    <t>0.3B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">240MB </t>
+  </si>
+  <si>
+    <t>340.65 ms</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1653,6 +1842,12 @@
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Google Sans"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -2096,7 +2291,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -2136,6 +2331,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2521,7 +2717,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A897CD1C-0E15-574E-9F3A-4CBFEDFF084C}">
-  <dimension ref="A1:V224"/>
+  <dimension ref="A1:V254"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="2" max="2" width="10.375" customWidth="1"/>
@@ -2536,70 +2732,70 @@
   <sheetData>
     <row r="1" spans="1:22"/>
     <row r="2" spans="1:22" ht="21">
-      <c r="A2" s="37" t="s">
+      <c r="A2" s="38" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="37" t="s">
+      <c r="B2" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="44" t="s">
+      <c r="C2" s="45" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="48" t="s">
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="49" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="49"/>
-      <c r="I2" s="49"/>
-      <c r="J2" s="49"/>
-      <c r="K2" s="49"/>
-      <c r="L2" s="49"/>
-      <c r="M2" s="49"/>
-      <c r="N2" s="50"/>
-      <c r="O2" s="42" t="s">
+      <c r="H2" s="50"/>
+      <c r="I2" s="50"/>
+      <c r="J2" s="50"/>
+      <c r="K2" s="50"/>
+      <c r="L2" s="50"/>
+      <c r="M2" s="50"/>
+      <c r="N2" s="51"/>
+      <c r="O2" s="43" t="s">
         <v>4</v>
       </c>
-      <c r="P2" s="42"/>
-      <c r="Q2" s="42"/>
-      <c r="R2" s="42"/>
-      <c r="S2" s="42"/>
-      <c r="T2" s="42"/>
-      <c r="U2" s="42"/>
-      <c r="V2" s="43"/>
+      <c r="P2" s="43"/>
+      <c r="Q2" s="43"/>
+      <c r="R2" s="43"/>
+      <c r="S2" s="43"/>
+      <c r="T2" s="43"/>
+      <c r="U2" s="43"/>
+      <c r="V2" s="44"/>
     </row>
     <row r="3" spans="1:22" ht="18.75">
-      <c r="A3" s="38"/>
-      <c r="B3" s="38"/>
-      <c r="C3" s="46"/>
-      <c r="D3" s="47"/>
-      <c r="E3" s="47"/>
-      <c r="F3" s="47"/>
-      <c r="G3" s="51"/>
-      <c r="H3" s="52"/>
-      <c r="I3" s="52"/>
-      <c r="J3" s="52"/>
-      <c r="K3" s="52"/>
-      <c r="L3" s="52"/>
-      <c r="M3" s="52"/>
-      <c r="N3" s="53"/>
-      <c r="O3" s="40" t="s">
+      <c r="A3" s="39"/>
+      <c r="B3" s="39"/>
+      <c r="C3" s="47"/>
+      <c r="D3" s="48"/>
+      <c r="E3" s="48"/>
+      <c r="F3" s="48"/>
+      <c r="G3" s="52"/>
+      <c r="H3" s="53"/>
+      <c r="I3" s="53"/>
+      <c r="J3" s="53"/>
+      <c r="K3" s="53"/>
+      <c r="L3" s="53"/>
+      <c r="M3" s="53"/>
+      <c r="N3" s="54"/>
+      <c r="O3" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="P3" s="40"/>
-      <c r="Q3" s="40"/>
-      <c r="R3" s="40" t="s">
+      <c r="P3" s="41"/>
+      <c r="Q3" s="41"/>
+      <c r="R3" s="41" t="s">
         <v>6</v>
       </c>
-      <c r="S3" s="40"/>
-      <c r="T3" s="40"/>
-      <c r="U3" s="40"/>
-      <c r="V3" s="41"/>
+      <c r="S3" s="41"/>
+      <c r="T3" s="41"/>
+      <c r="U3" s="41"/>
+      <c r="V3" s="42"/>
     </row>
     <row r="4" spans="1:22">
-      <c r="A4" s="39"/>
-      <c r="B4" s="39"/>
+      <c r="A4" s="40"/>
+      <c r="B4" s="40"/>
       <c r="C4" s="11" t="s">
         <v>7</v>
       </c>
@@ -13480,9 +13676,11 @@
       <c r="C213" s="12" t="s">
         <v>487</v>
       </c>
-      <c r="D213" s="2"/>
+      <c r="D213" s="2" t="s">
+        <v>488</v>
+      </c>
       <c r="E213" s="2" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="F213" s="2" t="s">
         <v>69</v>
@@ -13528,13 +13726,13 @@
         <v>393</v>
       </c>
       <c r="C214" s="12" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="D214" t="s">
         <v>409</v>
       </c>
       <c r="E214" s="2" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="F214" t="s">
         <v>69</v>
@@ -13580,7 +13778,7 @@
         <v>398</v>
       </c>
       <c r="C215" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="D215" t="s">
         <v>409</v>
@@ -13606,7 +13804,7 @@
         <v>0.37</v>
       </c>
       <c r="Q215" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="R215">
         <v>0.496</v>
@@ -13632,16 +13830,16 @@
         <v>367</v>
       </c>
       <c r="C216" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="D216" s="2" t="s">
         <v>53</v>
       </c>
       <c r="E216" s="2" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="F216" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="G216" s="23"/>
       <c r="H216" s="2"/>
@@ -13658,7 +13856,7 @@
         <v>0.40400000000000003</v>
       </c>
       <c r="Q216" s="2" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="R216" s="2">
         <v>0.52300000000000002</v>
@@ -13684,13 +13882,13 @@
         <v>393</v>
       </c>
       <c r="C217" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="D217" s="2" t="s">
         <v>477</v>
       </c>
       <c r="E217" s="2" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="F217" s="2" t="s">
         <v>69</v>
@@ -13736,13 +13934,13 @@
         <v>398</v>
       </c>
       <c r="C218" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="D218" t="s">
         <v>409</v>
       </c>
       <c r="E218" s="2" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="F218" s="2" t="s">
         <v>69</v>
@@ -13762,7 +13960,7 @@
         <v>0.624</v>
       </c>
       <c r="Q218" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="R218">
         <v>0.69899999999999995</v>
@@ -13788,13 +13986,13 @@
         <v>393</v>
       </c>
       <c r="C219" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="D219" s="2" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="E219" s="2" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="F219" s="2" t="s">
         <v>88</v>
@@ -13814,7 +14012,7 @@
         <v>0.624</v>
       </c>
       <c r="Q219" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="R219">
         <v>0.69899999999999995</v>
@@ -13840,7 +14038,7 @@
         <v>398</v>
       </c>
       <c r="C220" s="12" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="D220" t="s">
         <v>468</v>
@@ -13866,7 +14064,7 @@
         <v>0.48799999999999999</v>
       </c>
       <c r="Q220" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="R220">
         <v>0.59099999999999997</v>
@@ -13892,7 +14090,7 @@
         <v>393</v>
       </c>
       <c r="C221" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="D221" s="2" t="s">
         <v>376</v>
@@ -13918,7 +14116,7 @@
         <v>0.53</v>
       </c>
       <c r="Q221" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="R221">
         <v>0.624</v>
@@ -13944,7 +14142,7 @@
         <v>398</v>
       </c>
       <c r="C222" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="D222" s="2" t="s">
         <v>34</v>
@@ -13970,7 +14168,7 @@
         <v>0.60099999999999998</v>
       </c>
       <c r="Q222" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="R222">
         <v>0.68100000000000005</v>
@@ -13996,16 +14194,16 @@
         <v>367</v>
       </c>
       <c r="C223" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="D223" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="E223" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="F223" s="2" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="G223" s="23"/>
       <c r="H223" s="2"/>
@@ -14022,7 +14220,7 @@
         <v>0.34300000000000003</v>
       </c>
       <c r="Q223" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="R223">
         <v>0.45500000000000002</v>
@@ -14048,16 +14246,16 @@
         <v>367</v>
       </c>
       <c r="C224" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="D224" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="E224" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="F224" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="G224" s="23"/>
       <c r="O224">
@@ -14067,7 +14265,7 @@
         <v>0.23300000000000001</v>
       </c>
       <c r="Q224" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="R224">
         <v>0.33800000000000002</v>
@@ -14084,6 +14282,1230 @@
       <c r="V224">
         <v>0.30199999999999999</v>
       </c>
+    </row>
+    <row r="225" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A225" s="13">
+        <v>46322</v>
+      </c>
+      <c r="B225" s="10" t="s">
+        <v>393</v>
+      </c>
+      <c r="C225" t="s">
+        <v>523</v>
+      </c>
+      <c r="D225" t="s">
+        <v>409</v>
+      </c>
+      <c r="E225" s="2" t="s">
+        <v>524</v>
+      </c>
+      <c r="F225" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="G225" s="24"/>
+      <c r="H225" s="24"/>
+      <c r="I225" s="24"/>
+      <c r="J225" s="13"/>
+      <c r="K225" s="13"/>
+      <c r="L225" s="13"/>
+      <c r="M225" s="24"/>
+      <c r="N225" s="23"/>
+      <c r="O225">
+        <v>0.65100000000000002</v>
+      </c>
+      <c r="P225">
+        <v>0.623</v>
+      </c>
+      <c r="Q225" t="s">
+        <v>525</v>
+      </c>
+      <c r="R225">
+        <v>0.69899999999999995</v>
+      </c>
+      <c r="S225">
+        <v>0.54900000000000004</v>
+      </c>
+      <c r="T225">
+        <v>1</v>
+      </c>
+      <c r="U225">
+        <v>0.82399999999999995</v>
+      </c>
+      <c r="V225">
+        <v>0.59599999999999997</v>
+      </c>
+    </row>
+    <row r="226" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A226" s="13">
+        <v>46322</v>
+      </c>
+      <c r="B226" s="10" t="s">
+        <v>398</v>
+      </c>
+      <c r="C226" s="12" t="s">
+        <v>526</v>
+      </c>
+      <c r="D226" t="s">
+        <v>257</v>
+      </c>
+      <c r="E226" s="2" t="s">
+        <v>527</v>
+      </c>
+      <c r="F226" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="G226" s="13"/>
+      <c r="H226" s="24"/>
+      <c r="I226" s="24"/>
+      <c r="J226" s="13"/>
+      <c r="K226" s="23"/>
+      <c r="L226" s="13"/>
+      <c r="M226" s="24"/>
+      <c r="N226" s="13"/>
+      <c r="O226">
+        <v>0.89300000000000002</v>
+      </c>
+      <c r="P226">
+        <v>0.49099999999999999</v>
+      </c>
+      <c r="Q226" t="s">
+        <v>528</v>
+      </c>
+      <c r="R226">
+        <v>0.59299999999999997</v>
+      </c>
+      <c r="S226">
+        <v>0.60199999999999998</v>
+      </c>
+      <c r="T226">
+        <v>1</v>
+      </c>
+      <c r="U226">
+        <v>0.89200000000000002</v>
+      </c>
+      <c r="V226">
+        <v>0.61299999999999999</v>
+      </c>
+    </row>
+    <row r="227" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A227" s="13">
+        <v>46322</v>
+      </c>
+      <c r="B227" s="10" t="s">
+        <v>393</v>
+      </c>
+      <c r="C227" t="s">
+        <v>529</v>
+      </c>
+      <c r="D227" s="36" t="s">
+        <v>115</v>
+      </c>
+      <c r="E227" s="2" t="s">
+        <v>530</v>
+      </c>
+      <c r="F227" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="G227" s="13"/>
+      <c r="H227" s="24"/>
+      <c r="I227" s="24"/>
+      <c r="J227" s="13"/>
+      <c r="K227" s="23"/>
+      <c r="L227" s="13"/>
+      <c r="M227" s="24"/>
+      <c r="N227" s="13"/>
+      <c r="O227">
+        <v>0.83</v>
+      </c>
+      <c r="P227">
+        <v>0.45400000000000001</v>
+      </c>
+      <c r="Q227" t="s">
+        <v>531</v>
+      </c>
+      <c r="R227">
+        <v>0.56299999999999994</v>
+      </c>
+      <c r="S227">
+        <v>0.61199999999999999</v>
+      </c>
+      <c r="T227">
+        <v>0.90500000000000003</v>
+      </c>
+      <c r="U227">
+        <v>0.83799999999999997</v>
+      </c>
+      <c r="V227">
+        <v>0.56999999999999995</v>
+      </c>
+    </row>
+    <row r="228" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A228" s="13">
+        <v>46322</v>
+      </c>
+      <c r="B228" s="10" t="s">
+        <v>398</v>
+      </c>
+      <c r="C228" s="12" t="s">
+        <v>532</v>
+      </c>
+      <c r="D228" t="s">
+        <v>257</v>
+      </c>
+      <c r="E228" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="F228" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="G228" s="13"/>
+      <c r="H228" s="24"/>
+      <c r="I228" s="24"/>
+      <c r="J228" s="13"/>
+      <c r="K228" s="23"/>
+      <c r="L228" s="13"/>
+      <c r="M228" s="24"/>
+      <c r="N228" s="13"/>
+      <c r="O228">
+        <v>0.85699999999999998</v>
+      </c>
+      <c r="P228">
+        <v>0.497</v>
+      </c>
+      <c r="Q228" t="s">
+        <v>533</v>
+      </c>
+      <c r="R228">
+        <v>0.59799999999999998</v>
+      </c>
+      <c r="S228">
+        <v>0.59599999999999997</v>
+      </c>
+      <c r="T228">
+        <v>1</v>
+      </c>
+      <c r="U228">
+        <v>0.88300000000000001</v>
+      </c>
+      <c r="V228">
+        <v>0.60499999999999998</v>
+      </c>
+    </row>
+    <row r="229" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A229" s="13">
+        <v>46322</v>
+      </c>
+      <c r="B229" s="10" t="s">
+        <v>393</v>
+      </c>
+      <c r="C229" s="12" t="s">
+        <v>534</v>
+      </c>
+      <c r="D229" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="E229" s="2" t="s">
+        <v>535</v>
+      </c>
+      <c r="F229" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="G229" s="13"/>
+      <c r="H229" s="24"/>
+      <c r="I229" s="24"/>
+      <c r="J229" s="13"/>
+      <c r="K229" s="23"/>
+      <c r="L229" s="13"/>
+      <c r="M229" s="24"/>
+      <c r="N229" s="13"/>
+      <c r="O229">
+        <v>0.85199999999999998</v>
+      </c>
+      <c r="P229">
+        <v>0.54600000000000004</v>
+      </c>
+      <c r="Q229" t="s">
+        <v>536</v>
+      </c>
+      <c r="R229">
+        <v>0.63700000000000001</v>
+      </c>
+      <c r="S229">
+        <v>0.58699999999999997</v>
+      </c>
+      <c r="T229">
+        <v>1</v>
+      </c>
+      <c r="U229">
+        <v>0.88900000000000001</v>
+      </c>
+      <c r="V229">
+        <v>0.61899999999999999</v>
+      </c>
+    </row>
+    <row r="230" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A230" s="13">
+        <v>46322</v>
+      </c>
+      <c r="B230" s="10" t="s">
+        <v>398</v>
+      </c>
+      <c r="C230" s="12" t="s">
+        <v>537</v>
+      </c>
+      <c r="D230" t="s">
+        <v>257</v>
+      </c>
+      <c r="E230" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="F230" t="s">
+        <v>538</v>
+      </c>
+      <c r="G230" s="13"/>
+      <c r="H230" s="23"/>
+      <c r="I230" s="24"/>
+      <c r="J230" s="13"/>
+      <c r="K230" s="13"/>
+      <c r="L230" s="13"/>
+      <c r="M230" s="24"/>
+      <c r="N230" s="13"/>
+      <c r="O230">
+        <v>0.72199999999999998</v>
+      </c>
+      <c r="P230">
+        <v>0.69699999999999995</v>
+      </c>
+      <c r="Q230" t="s">
+        <v>539</v>
+      </c>
+      <c r="R230">
+        <v>0.75800000000000001</v>
+      </c>
+      <c r="S230">
+        <v>0.52400000000000002</v>
+      </c>
+      <c r="T230">
+        <v>0.82</v>
+      </c>
+      <c r="U230">
+        <v>0.94199999999999995</v>
+      </c>
+      <c r="V230">
+        <v>0.61699999999999999</v>
+      </c>
+    </row>
+    <row r="231" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A231" s="13">
+        <v>46322</v>
+      </c>
+      <c r="B231" s="10" t="s">
+        <v>393</v>
+      </c>
+      <c r="C231" s="12" t="s">
+        <v>446</v>
+      </c>
+      <c r="D231" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="E231" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="F231" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="G231" s="13"/>
+      <c r="H231" s="24"/>
+      <c r="I231" s="23"/>
+      <c r="J231" s="13"/>
+      <c r="K231" s="13"/>
+      <c r="L231" s="13"/>
+      <c r="M231" s="24"/>
+      <c r="N231" s="13"/>
+      <c r="O231">
+        <v>0.82099999999999995</v>
+      </c>
+      <c r="P231">
+        <v>0.64300000000000002</v>
+      </c>
+      <c r="Q231" t="s">
+        <v>540</v>
+      </c>
+      <c r="R231">
+        <v>0.71499999999999997</v>
+      </c>
+      <c r="S231">
+        <v>0.54100000000000004</v>
+      </c>
+      <c r="T231">
+        <v>0.96299999999999997</v>
+      </c>
+      <c r="U231">
+        <v>0.92800000000000005</v>
+      </c>
+      <c r="V231">
+        <v>0.63300000000000001</v>
+      </c>
+    </row>
+    <row r="232" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A232" s="13">
+        <v>46322</v>
+      </c>
+      <c r="B232" s="10" t="s">
+        <v>398</v>
+      </c>
+      <c r="C232" s="12" t="s">
+        <v>541</v>
+      </c>
+      <c r="D232" s="2" t="s">
+        <v>542</v>
+      </c>
+      <c r="E232" s="2" t="s">
+        <v>543</v>
+      </c>
+      <c r="F232" s="37" t="s">
+        <v>544</v>
+      </c>
+      <c r="G232" s="13"/>
+      <c r="H232" s="24"/>
+      <c r="I232" s="24"/>
+      <c r="J232" s="13"/>
+      <c r="K232" s="13"/>
+      <c r="L232" s="23"/>
+      <c r="M232" s="24"/>
+      <c r="N232" s="13"/>
+      <c r="O232">
+        <v>0.77500000000000002</v>
+      </c>
+      <c r="P232">
+        <v>0.58499999999999996</v>
+      </c>
+      <c r="Q232" t="s">
+        <v>545</v>
+      </c>
+      <c r="R232">
+        <v>0.66800000000000004</v>
+      </c>
+      <c r="S232">
+        <v>0.56499999999999995</v>
+      </c>
+      <c r="T232">
+        <v>0.90200000000000002</v>
+      </c>
+      <c r="U232">
+        <v>0.877</v>
+      </c>
+      <c r="V232">
+        <v>0.59199999999999997</v>
+      </c>
+    </row>
+    <row r="233" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A233" s="13">
+        <v>46322</v>
+      </c>
+      <c r="B233" s="10" t="s">
+        <v>393</v>
+      </c>
+      <c r="C233" s="12" t="s">
+        <v>546</v>
+      </c>
+      <c r="D233" s="2" t="s">
+        <v>542</v>
+      </c>
+      <c r="E233" s="2" t="s">
+        <v>547</v>
+      </c>
+      <c r="F233" s="2" t="s">
+        <v>548</v>
+      </c>
+      <c r="G233" s="13"/>
+      <c r="H233" s="24"/>
+      <c r="I233" s="24"/>
+      <c r="J233" s="13"/>
+      <c r="K233" s="13"/>
+      <c r="L233" s="13"/>
+      <c r="M233" s="23"/>
+      <c r="N233" s="13"/>
+      <c r="O233">
+        <v>0.70499999999999996</v>
+      </c>
+      <c r="P233">
+        <v>0.60899999999999999</v>
+      </c>
+      <c r="Q233" t="s">
+        <v>549</v>
+      </c>
+      <c r="R233">
+        <v>0.68700000000000006</v>
+      </c>
+      <c r="S233">
+        <v>0.55500000000000005</v>
+      </c>
+      <c r="T233">
+        <v>1</v>
+      </c>
+      <c r="U233">
+        <v>0.88</v>
+      </c>
+      <c r="V233">
+        <v>0.60099999999999998</v>
+      </c>
+    </row>
+    <row r="234" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A234" s="13">
+        <v>46322</v>
+      </c>
+      <c r="B234" s="10" t="s">
+        <v>398</v>
+      </c>
+      <c r="C234" s="12" t="s">
+        <v>550</v>
+      </c>
+      <c r="D234" s="2" t="s">
+        <v>542</v>
+      </c>
+      <c r="E234" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="F234" t="s">
+        <v>552</v>
+      </c>
+      <c r="G234" s="23"/>
+      <c r="H234" s="24"/>
+      <c r="I234" s="24"/>
+      <c r="J234" s="13"/>
+      <c r="K234" s="13"/>
+      <c r="L234" s="13"/>
+      <c r="M234" s="24"/>
+      <c r="N234" s="13"/>
+      <c r="O234">
+        <v>0.3</v>
+      </c>
+      <c r="P234">
+        <v>0.48499999999999999</v>
+      </c>
+      <c r="Q234" t="s">
+        <v>553</v>
+      </c>
+      <c r="R234">
+        <v>0.54800000000000004</v>
+      </c>
+      <c r="S234">
+        <v>0.60099999999999998</v>
+      </c>
+      <c r="T234">
+        <v>1</v>
+      </c>
+      <c r="U234">
+        <v>0.66600000000000004</v>
+      </c>
+      <c r="V234">
+        <v>0.46</v>
+      </c>
+    </row>
+    <row r="235" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A235" s="13">
+        <v>46322</v>
+      </c>
+      <c r="B235" s="10" t="s">
+        <v>393</v>
+      </c>
+      <c r="C235" s="12" t="s">
+        <v>554</v>
+      </c>
+      <c r="D235" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E235" t="s">
+        <v>197</v>
+      </c>
+      <c r="F235" t="s">
+        <v>555</v>
+      </c>
+      <c r="G235" s="13"/>
+      <c r="H235" s="24"/>
+      <c r="I235" s="23"/>
+      <c r="J235" s="13"/>
+      <c r="K235" s="13"/>
+      <c r="L235" s="13"/>
+      <c r="M235" s="24"/>
+      <c r="N235" s="13"/>
+      <c r="O235">
+        <v>0.88100000000000001</v>
+      </c>
+      <c r="P235">
+        <v>0.65</v>
+      </c>
+      <c r="Q235" t="s">
+        <v>556</v>
+      </c>
+      <c r="R235">
+        <v>0.72</v>
+      </c>
+      <c r="S235">
+        <v>0.54100000000000004</v>
+      </c>
+      <c r="T235">
+        <v>0.878</v>
+      </c>
+      <c r="U235">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="V235">
+        <v>0.63100000000000001</v>
+      </c>
+    </row>
+    <row r="236" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A236" s="13">
+        <v>46322</v>
+      </c>
+      <c r="B236" s="10" t="s">
+        <v>398</v>
+      </c>
+      <c r="C236" s="12" t="s">
+        <v>557</v>
+      </c>
+      <c r="D236" s="2" t="s">
+        <v>558</v>
+      </c>
+      <c r="E236" t="s">
+        <v>559</v>
+      </c>
+      <c r="F236" s="2" t="s">
+        <v>555</v>
+      </c>
+      <c r="G236" s="13"/>
+      <c r="H236" s="24"/>
+      <c r="I236" s="24"/>
+      <c r="J236" s="13"/>
+      <c r="K236" s="23"/>
+      <c r="L236" s="13"/>
+      <c r="M236" s="24"/>
+      <c r="N236" s="13"/>
+      <c r="O236">
+        <v>0.78</v>
+      </c>
+      <c r="P236">
+        <v>0.51700000000000002</v>
+      </c>
+      <c r="Q236" t="s">
+        <v>560</v>
+      </c>
+      <c r="R236">
+        <v>0.61399999999999999</v>
+      </c>
+      <c r="S236">
+        <v>0.58899999999999997</v>
+      </c>
+      <c r="T236">
+        <v>1</v>
+      </c>
+      <c r="U236">
+        <v>0.86199999999999999</v>
+      </c>
+      <c r="V236">
+        <v>0.59299999999999997</v>
+      </c>
+    </row>
+    <row r="237" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A237" s="13">
+        <v>46322</v>
+      </c>
+      <c r="B237" s="10" t="s">
+        <v>393</v>
+      </c>
+      <c r="C237" s="12" t="s">
+        <v>561</v>
+      </c>
+      <c r="D237" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="E237" s="2" t="s">
+        <v>562</v>
+      </c>
+      <c r="F237" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="G237" s="13"/>
+      <c r="H237" s="24"/>
+      <c r="I237" s="24"/>
+      <c r="J237" s="13"/>
+      <c r="K237" s="13"/>
+      <c r="L237" s="13"/>
+      <c r="M237" s="24"/>
+      <c r="N237" s="23"/>
+      <c r="O237">
+        <v>0.78</v>
+      </c>
+      <c r="P237">
+        <v>0.58799999999999997</v>
+      </c>
+      <c r="Q237" t="s">
+        <v>563</v>
+      </c>
+      <c r="R237">
+        <v>0.67</v>
+      </c>
+      <c r="S237">
+        <v>0.57099999999999995</v>
+      </c>
+      <c r="T237">
+        <v>1</v>
+      </c>
+      <c r="U237">
+        <v>0.84499999999999997</v>
+      </c>
+      <c r="V237">
+        <v>0.60199999999999998</v>
+      </c>
+    </row>
+    <row r="238" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A238" s="13">
+        <v>46322</v>
+      </c>
+      <c r="B238" s="10" t="s">
+        <v>398</v>
+      </c>
+      <c r="C238" s="12" t="s">
+        <v>564</v>
+      </c>
+      <c r="D238" s="2" t="s">
+        <v>565</v>
+      </c>
+      <c r="E238" s="2" t="s">
+        <v>566</v>
+      </c>
+      <c r="F238" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="G238" s="13"/>
+      <c r="H238" s="24"/>
+      <c r="I238" s="24"/>
+      <c r="J238" s="23"/>
+      <c r="K238" s="13"/>
+      <c r="L238" s="13"/>
+      <c r="M238" s="24"/>
+      <c r="N238" s="13"/>
+      <c r="O238">
+        <v>0.75800000000000001</v>
+      </c>
+      <c r="P238">
+        <v>0.66300000000000003</v>
+      </c>
+      <c r="Q238" t="s">
+        <v>567</v>
+      </c>
+      <c r="R238">
+        <v>0.73</v>
+      </c>
+      <c r="S238">
+        <v>0.53500000000000003</v>
+      </c>
+      <c r="T238">
+        <v>0.93700000000000006</v>
+      </c>
+      <c r="U238">
+        <v>0.89800000000000002</v>
+      </c>
+      <c r="V238">
+        <v>0.621</v>
+      </c>
+    </row>
+    <row r="239" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A239" s="13">
+        <v>46322</v>
+      </c>
+      <c r="B239" s="10" t="s">
+        <v>393</v>
+      </c>
+      <c r="C239" s="12" t="s">
+        <v>568</v>
+      </c>
+      <c r="D239" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="E239" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="F239" s="2" t="s">
+        <v>569</v>
+      </c>
+      <c r="G239" s="13"/>
+      <c r="H239" s="24"/>
+      <c r="I239" s="13"/>
+      <c r="J239" s="13"/>
+      <c r="K239" s="13"/>
+      <c r="L239" s="23"/>
+      <c r="M239" s="24"/>
+      <c r="N239" s="13"/>
+      <c r="O239">
+        <v>0.76</v>
+      </c>
+      <c r="P239">
+        <v>0.60899999999999999</v>
+      </c>
+      <c r="Q239" t="s">
+        <v>570</v>
+      </c>
+      <c r="R239">
+        <v>0.68799999999999994</v>
+      </c>
+      <c r="S239">
+        <v>0.55900000000000005</v>
+      </c>
+      <c r="T239">
+        <v>0.85</v>
+      </c>
+      <c r="U239">
+        <v>0.878</v>
+      </c>
+      <c r="V239">
+        <v>0.59499999999999997</v>
+      </c>
+    </row>
+    <row r="240" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A240" s="13">
+        <v>46322</v>
+      </c>
+      <c r="B240" s="10" t="s">
+        <v>398</v>
+      </c>
+      <c r="C240" s="12" t="s">
+        <v>571</v>
+      </c>
+      <c r="D240" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E240" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="F240" s="2" t="s">
+        <v>572</v>
+      </c>
+      <c r="G240" s="13"/>
+      <c r="H240" s="24"/>
+      <c r="I240" s="24"/>
+      <c r="J240" s="13"/>
+      <c r="K240" s="13"/>
+      <c r="L240" s="13"/>
+      <c r="M240" s="23"/>
+      <c r="N240" s="13"/>
+      <c r="O240">
+        <v>0.78</v>
+      </c>
+      <c r="P240">
+        <v>0.39500000000000002</v>
+      </c>
+      <c r="Q240" t="s">
+        <v>573</v>
+      </c>
+      <c r="R240">
+        <v>0.46600000000000003</v>
+      </c>
+      <c r="S240">
+        <v>0.624</v>
+      </c>
+      <c r="T240">
+        <v>1</v>
+      </c>
+      <c r="U240">
+        <v>0.82099999999999995</v>
+      </c>
+      <c r="V240">
+        <v>0.54600000000000004</v>
+      </c>
+    </row>
+    <row r="241" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A241" s="13">
+        <v>46322</v>
+      </c>
+      <c r="B241" s="10" t="s">
+        <v>393</v>
+      </c>
+      <c r="C241" t="s">
+        <v>574</v>
+      </c>
+      <c r="D241" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="E241" s="2" t="s">
+        <v>575</v>
+      </c>
+      <c r="F241" t="s">
+        <v>69</v>
+      </c>
+      <c r="G241" s="13"/>
+      <c r="H241" s="24"/>
+      <c r="I241" s="24"/>
+      <c r="J241" s="13"/>
+      <c r="K241" s="13"/>
+      <c r="L241" s="13"/>
+      <c r="M241" s="24"/>
+      <c r="N241" s="23"/>
+      <c r="O241">
+        <v>0.60399999999999998</v>
+      </c>
+      <c r="P241">
+        <v>0.55100000000000005</v>
+      </c>
+      <c r="Q241" t="s">
+        <v>576</v>
+      </c>
+      <c r="R241">
+        <v>0.64100000000000001</v>
+      </c>
+      <c r="S241">
+        <v>0.57799999999999996</v>
+      </c>
+      <c r="T241">
+        <v>1</v>
+      </c>
+      <c r="U241">
+        <v>0.88100000000000001</v>
+      </c>
+      <c r="V241">
+        <v>0.56899999999999995</v>
+      </c>
+    </row>
+    <row r="242" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A242" s="13">
+        <v>46322</v>
+      </c>
+      <c r="B242" s="10" t="s">
+        <v>398</v>
+      </c>
+      <c r="C242" t="s">
+        <v>577</v>
+      </c>
+      <c r="D242" s="2" t="s">
+        <v>578</v>
+      </c>
+      <c r="E242" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="F242" t="s">
+        <v>69</v>
+      </c>
+      <c r="G242" s="23"/>
+      <c r="H242" s="24"/>
+      <c r="I242" s="24"/>
+      <c r="J242" s="13"/>
+      <c r="K242" s="13"/>
+      <c r="L242" s="13"/>
+      <c r="M242" s="24"/>
+      <c r="N242" s="13"/>
+      <c r="O242">
+        <v>0.26800000000000002</v>
+      </c>
+      <c r="P242">
+        <v>0.32</v>
+      </c>
+      <c r="Q242" t="s">
+        <v>580</v>
+      </c>
+      <c r="R242">
+        <v>0.436</v>
+      </c>
+      <c r="S242">
+        <v>0.65500000000000003</v>
+      </c>
+      <c r="T242">
+        <v>1</v>
+      </c>
+      <c r="U242">
+        <v>0.69499999999999995</v>
+      </c>
+      <c r="V242">
+        <v>0.41699999999999998</v>
+      </c>
+    </row>
+    <row r="243" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A243" s="13"/>
+      <c r="B243" s="10"/>
+      <c r="C243" s="12"/>
+      <c r="D243" s="2"/>
+      <c r="E243" s="2"/>
+      <c r="F243" s="2"/>
+      <c r="G243" s="13"/>
+      <c r="H243" s="24"/>
+      <c r="I243" s="24"/>
+      <c r="J243" s="13"/>
+      <c r="K243" s="13"/>
+      <c r="L243" s="13"/>
+      <c r="M243" s="24"/>
+      <c r="N243" s="13"/>
+      <c r="O243" s="10"/>
+      <c r="P243" s="10"/>
+      <c r="Q243" s="10"/>
+      <c r="R243" s="10"/>
+      <c r="S243" s="10"/>
+      <c r="T243" s="10"/>
+      <c r="U243" s="10"/>
+      <c r="V243" s="6"/>
+    </row>
+    <row r="244" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A244" s="13"/>
+      <c r="B244" s="10"/>
+      <c r="C244" s="12"/>
+      <c r="D244" s="2"/>
+      <c r="E244" s="2"/>
+      <c r="F244" s="2"/>
+      <c r="G244" s="13"/>
+      <c r="H244" s="24"/>
+      <c r="I244" s="24"/>
+      <c r="J244" s="13"/>
+      <c r="K244" s="13"/>
+      <c r="L244" s="13"/>
+      <c r="M244" s="24"/>
+      <c r="N244" s="13"/>
+      <c r="O244" s="10"/>
+      <c r="P244" s="10"/>
+      <c r="Q244" s="10"/>
+      <c r="R244" s="10"/>
+      <c r="S244" s="10"/>
+      <c r="T244" s="10"/>
+      <c r="U244" s="10"/>
+      <c r="V244" s="6"/>
+    </row>
+    <row r="245" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A245" s="13"/>
+      <c r="B245" s="10"/>
+      <c r="C245" s="12"/>
+      <c r="D245" s="2"/>
+      <c r="E245" s="2"/>
+      <c r="F245" s="2"/>
+      <c r="G245" s="13"/>
+      <c r="H245" s="24"/>
+      <c r="I245" s="24"/>
+      <c r="J245" s="13"/>
+      <c r="K245" s="13"/>
+      <c r="L245" s="13"/>
+      <c r="M245" s="24"/>
+      <c r="N245" s="13"/>
+      <c r="O245" s="10"/>
+      <c r="P245" s="10"/>
+      <c r="Q245" s="10"/>
+      <c r="R245" s="10"/>
+      <c r="S245" s="10"/>
+      <c r="T245" s="10"/>
+      <c r="U245" s="10"/>
+      <c r="V245" s="6"/>
+    </row>
+    <row r="246" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A246" s="13"/>
+      <c r="B246" s="10"/>
+      <c r="C246" s="12"/>
+      <c r="D246" s="2"/>
+      <c r="E246" s="2"/>
+      <c r="F246" s="2"/>
+      <c r="G246" s="13"/>
+      <c r="H246" s="24"/>
+      <c r="I246" s="24"/>
+      <c r="J246" s="13"/>
+      <c r="K246" s="13"/>
+      <c r="L246" s="13"/>
+      <c r="M246" s="24"/>
+      <c r="N246" s="13"/>
+      <c r="O246" s="10"/>
+      <c r="P246" s="10"/>
+      <c r="Q246" s="10"/>
+      <c r="R246" s="10"/>
+      <c r="S246" s="10"/>
+      <c r="T246" s="10"/>
+      <c r="U246" s="10"/>
+      <c r="V246" s="6"/>
+    </row>
+    <row r="247" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A247" s="13"/>
+      <c r="B247" s="10"/>
+      <c r="C247" s="12"/>
+      <c r="D247" s="2"/>
+      <c r="E247" s="2"/>
+      <c r="F247" s="2"/>
+      <c r="G247" s="13"/>
+      <c r="H247" s="24"/>
+      <c r="I247" s="24"/>
+      <c r="J247" s="13"/>
+      <c r="K247" s="13"/>
+      <c r="L247" s="13"/>
+      <c r="M247" s="24"/>
+      <c r="N247" s="13"/>
+      <c r="O247" s="10"/>
+      <c r="P247" s="10"/>
+      <c r="Q247" s="10"/>
+      <c r="R247" s="10"/>
+      <c r="S247" s="10"/>
+      <c r="T247" s="10"/>
+      <c r="U247" s="10"/>
+      <c r="V247" s="6"/>
+    </row>
+    <row r="248" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A248" s="13"/>
+      <c r="B248" s="10"/>
+      <c r="C248" s="12"/>
+      <c r="D248" s="2"/>
+      <c r="E248" s="2"/>
+      <c r="F248" s="2"/>
+      <c r="G248" s="13"/>
+      <c r="H248" s="24"/>
+      <c r="I248" s="24"/>
+      <c r="J248" s="13"/>
+      <c r="K248" s="13"/>
+      <c r="L248" s="13"/>
+      <c r="M248" s="24"/>
+      <c r="N248" s="13"/>
+      <c r="O248" s="10"/>
+      <c r="P248" s="10"/>
+      <c r="Q248" s="10"/>
+      <c r="R248" s="10"/>
+      <c r="S248" s="10"/>
+      <c r="T248" s="10"/>
+      <c r="U248" s="10"/>
+      <c r="V248" s="6"/>
+    </row>
+    <row r="249" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A249" s="13"/>
+      <c r="B249" s="10"/>
+      <c r="C249" s="12"/>
+      <c r="D249" s="2"/>
+      <c r="E249" s="2"/>
+      <c r="F249" s="2"/>
+      <c r="G249" s="13"/>
+      <c r="H249" s="24"/>
+      <c r="I249" s="24"/>
+      <c r="J249" s="13"/>
+      <c r="K249" s="13"/>
+      <c r="L249" s="13"/>
+      <c r="M249" s="24"/>
+      <c r="N249" s="13"/>
+      <c r="O249" s="10"/>
+      <c r="P249" s="10"/>
+      <c r="Q249" s="10"/>
+      <c r="R249" s="10"/>
+      <c r="S249" s="10"/>
+      <c r="T249" s="10"/>
+      <c r="U249" s="10"/>
+      <c r="V249" s="6"/>
+    </row>
+    <row r="250" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A250" s="13"/>
+      <c r="B250" s="10"/>
+      <c r="C250" s="12"/>
+      <c r="D250" s="2"/>
+      <c r="E250" s="2"/>
+      <c r="F250" s="2"/>
+      <c r="G250" s="13"/>
+      <c r="H250" s="24"/>
+      <c r="I250" s="24"/>
+      <c r="J250" s="13"/>
+      <c r="K250" s="13"/>
+      <c r="L250" s="13"/>
+      <c r="M250" s="24"/>
+      <c r="N250" s="13"/>
+      <c r="O250" s="10"/>
+      <c r="P250" s="10"/>
+      <c r="Q250" s="10"/>
+      <c r="R250" s="10"/>
+      <c r="S250" s="10"/>
+      <c r="T250" s="10"/>
+      <c r="U250" s="10"/>
+      <c r="V250" s="6"/>
+    </row>
+    <row r="251" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A251" s="13"/>
+      <c r="B251" s="10"/>
+      <c r="C251" s="12"/>
+      <c r="D251" s="2"/>
+      <c r="E251" s="2"/>
+      <c r="F251" s="2"/>
+      <c r="G251" s="13"/>
+      <c r="H251" s="24"/>
+      <c r="I251" s="24"/>
+      <c r="J251" s="13"/>
+      <c r="K251" s="13"/>
+      <c r="L251" s="13"/>
+      <c r="M251" s="24"/>
+      <c r="N251" s="13"/>
+      <c r="O251" s="10"/>
+      <c r="P251" s="10"/>
+      <c r="Q251" s="10"/>
+      <c r="R251" s="10"/>
+      <c r="S251" s="10"/>
+      <c r="T251" s="10"/>
+      <c r="U251" s="10"/>
+      <c r="V251" s="6"/>
+    </row>
+    <row r="252" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A252" s="13"/>
+      <c r="B252" s="10"/>
+      <c r="C252" s="12"/>
+      <c r="D252" s="2"/>
+      <c r="E252" s="2"/>
+      <c r="F252" s="2"/>
+      <c r="G252" s="13"/>
+      <c r="H252" s="24"/>
+      <c r="I252" s="24"/>
+      <c r="J252" s="13"/>
+      <c r="K252" s="13"/>
+      <c r="L252" s="13"/>
+      <c r="M252" s="24"/>
+      <c r="N252" s="13"/>
+      <c r="O252" s="10"/>
+      <c r="P252" s="10"/>
+      <c r="Q252" s="10"/>
+      <c r="R252" s="10"/>
+      <c r="S252" s="10"/>
+      <c r="T252" s="10"/>
+      <c r="U252" s="10"/>
+      <c r="V252" s="6"/>
+    </row>
+    <row r="253" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A253" s="13"/>
+      <c r="B253" s="10"/>
+      <c r="C253" s="12"/>
+      <c r="D253" s="2"/>
+      <c r="E253" s="2"/>
+      <c r="F253" s="2"/>
+      <c r="G253" s="13"/>
+      <c r="H253" s="24"/>
+      <c r="I253" s="24"/>
+      <c r="J253" s="13"/>
+      <c r="K253" s="13"/>
+      <c r="L253" s="13"/>
+      <c r="M253" s="24"/>
+      <c r="N253" s="13"/>
+      <c r="O253" s="10"/>
+      <c r="P253" s="10"/>
+      <c r="Q253" s="10"/>
+      <c r="R253" s="10"/>
+      <c r="S253" s="10"/>
+      <c r="T253" s="10"/>
+      <c r="U253" s="10"/>
+      <c r="V253" s="6"/>
+    </row>
+    <row r="254" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A254" s="13"/>
+      <c r="B254" s="10"/>
+      <c r="C254" s="12"/>
+      <c r="D254" s="2"/>
+      <c r="E254" s="2"/>
+      <c r="F254" s="2"/>
+      <c r="G254" s="13"/>
+      <c r="H254" s="24"/>
+      <c r="I254" s="24"/>
+      <c r="J254" s="13"/>
+      <c r="K254" s="13"/>
+      <c r="L254" s="13"/>
+      <c r="M254" s="24"/>
+      <c r="N254" s="13"/>
+      <c r="O254" s="10"/>
+      <c r="P254" s="10"/>
+      <c r="Q254" s="10"/>
+      <c r="R254" s="10"/>
+      <c r="S254" s="10"/>
+      <c r="T254" s="10"/>
+      <c r="U254" s="10"/>
+      <c r="V254" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>

<commit_message>
responsvie fixed and some minor changes in landing page
</commit_message>
<xml_diff>
--- a/scratch/tracker.xlsx
+++ b/scratch/tracker.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30621"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30619"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://drpinnacle-my.sharepoint.com/personal/vish_drpinnacle_com/Documents/Projects/openvals/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4244" documentId="8_{F24D4BFB-FFC1-BD42-9143-22F6B790B9D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C43EDE8A-B74A-4D47-BC10-02FE8F00520B}"/>
+  <xr:revisionPtr revIDLastSave="4258" documentId="8_{F24D4BFB-FFC1-BD42-9143-22F6B790B9D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C02618C9-4EC3-426C-B10F-4D42C33DC25B}"/>
   <bookViews>
     <workbookView xWindow="3960" yWindow="2780" windowWidth="28040" windowHeight="17180" xr2:uid="{BEF502B7-096A-F24C-A77D-ED0F5F38F7FE}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1438" uniqueCount="581">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1443" uniqueCount="584">
   <si>
     <t>Date</t>
   </si>
@@ -1472,7 +1472,7 @@
     <t>678.99 ms</t>
   </si>
   <si>
-    <t xml:space="preserve"> gemma4:e2b</t>
+    <t>gemma4:e2b</t>
   </si>
   <si>
     <t>2B</t>
@@ -1484,7 +1484,7 @@
     <t>5721.52 ms</t>
   </si>
   <si>
-    <t xml:space="preserve"> deepcoder:1.5b</t>
+    <t>deepcoder:1.5b</t>
   </si>
   <si>
     <t>1.5B</t>
@@ -1748,7 +1748,7 @@
     <t>6113.64 ms</t>
   </si>
   <si>
-    <t xml:space="preserve"> gemma2:2b</t>
+    <t>gemma2:2b</t>
   </si>
   <si>
     <t>2.2b</t>
@@ -1797,6 +1797,15 @@
   </si>
   <si>
     <t>340.65 ms</t>
+  </si>
+  <si>
+    <t>blueishai/anant-base:q4</t>
+  </si>
+  <si>
+    <t>1.12 GB</t>
+  </si>
+  <si>
+    <t>970.50 ms</t>
   </si>
 </sst>
 </file>
@@ -15220,11 +15229,21 @@
       </c>
     </row>
     <row r="243" spans="1:22" ht="15.75" customHeight="1">
-      <c r="A243" s="13"/>
-      <c r="B243" s="10"/>
-      <c r="C243" s="12"/>
-      <c r="D243" s="2"/>
-      <c r="E243" s="2"/>
+      <c r="A243" s="13">
+        <v>46323</v>
+      </c>
+      <c r="B243" s="10" t="s">
+        <v>393</v>
+      </c>
+      <c r="C243" t="s">
+        <v>581</v>
+      </c>
+      <c r="D243" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="E243" s="2" t="s">
+        <v>582</v>
+      </c>
       <c r="F243" s="2"/>
       <c r="G243" s="13"/>
       <c r="H243" s="24"/>
@@ -15233,15 +15252,31 @@
       <c r="K243" s="13"/>
       <c r="L243" s="13"/>
       <c r="M243" s="24"/>
-      <c r="N243" s="13"/>
-      <c r="O243" s="10"/>
-      <c r="P243" s="10"/>
-      <c r="Q243" s="10"/>
-      <c r="R243" s="10"/>
-      <c r="S243" s="10"/>
-      <c r="T243" s="10"/>
-      <c r="U243" s="10"/>
-      <c r="V243" s="6"/>
+      <c r="N243" s="23"/>
+      <c r="O243">
+        <v>0.89700000000000002</v>
+      </c>
+      <c r="P243">
+        <v>0.76800000000000002</v>
+      </c>
+      <c r="Q243" t="s">
+        <v>583</v>
+      </c>
+      <c r="R243">
+        <v>0.66500000000000004</v>
+      </c>
+      <c r="S243">
+        <v>0.49099999999999999</v>
+      </c>
+      <c r="T243">
+        <v>1</v>
+      </c>
+      <c r="U243">
+        <v>0.876</v>
+      </c>
+      <c r="V243">
+        <v>0.67200000000000004</v>
+      </c>
     </row>
     <row r="244" spans="1:22" ht="15.75" customHeight="1">
       <c r="A244" s="13"/>

</xml_diff>

<commit_message>
UI & UX changes and fixed responsive issuse.
</commit_message>
<xml_diff>
--- a/scratch/tracker.xlsx
+++ b/scratch/tracker.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30619"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30621"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://drpinnacle-my.sharepoint.com/personal/vish_drpinnacle_com/Documents/Projects/openvals/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4551" documentId="8_{F24D4BFB-FFC1-BD42-9143-22F6B790B9D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{25252688-7057-4D7B-839D-20A3D7DE6668}"/>
+  <xr:revisionPtr revIDLastSave="4634" documentId="8_{F24D4BFB-FFC1-BD42-9143-22F6B790B9D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A456466-3883-4ED7-9DA2-CE3E8082B723}"/>
   <bookViews>
     <workbookView xWindow="3960" yWindow="2780" windowWidth="28040" windowHeight="17180" xr2:uid="{BEF502B7-096A-F24C-A77D-ED0F5F38F7FE}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1629" uniqueCount="671">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1672" uniqueCount="693">
   <si>
     <t>Date</t>
   </si>
@@ -2067,6 +2067,72 @@
   </si>
   <si>
     <t>4366.12 ms</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> MeetSolanki/MeetAISmall</t>
+  </si>
+  <si>
+    <t>0.7b</t>
+  </si>
+  <si>
+    <t>523 MB</t>
+  </si>
+  <si>
+    <t>1838.74 ms</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> tulu3</t>
+  </si>
+  <si>
+    <t>8b</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 4.9 GB</t>
+  </si>
+  <si>
+    <t>16814.81 ms</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> hf.co/mradermacher/Yi-Coder-1.5B-Chat-GGUF:Q4_K_M</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 963 MB</t>
+  </si>
+  <si>
+    <t>2509.01 ms</t>
+  </si>
+  <si>
+    <t>granite-3.3-2b-instruct-GGUF:Q4_K_M</t>
+  </si>
+  <si>
+    <t>6488.13 ms</t>
+  </si>
+  <si>
+    <t>MeetSolanki/MeetAISmall</t>
+  </si>
+  <si>
+    <t>241 MB</t>
+  </si>
+  <si>
+    <t>2193.75 ms</t>
+  </si>
+  <si>
+    <t>GRAFT-1B</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 971 MB</t>
+  </si>
+  <si>
+    <t>2087.55 ms</t>
+  </si>
+  <si>
+    <t>Granite 4.0 H-1B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">901 MB  </t>
+  </si>
+  <si>
+    <t>6533.02 ms</t>
   </si>
 </sst>
 </file>
@@ -2987,7 +3053,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A897CD1C-0E15-574E-9F3A-4CBFEDFF084C}">
-  <dimension ref="A1:V276"/>
+  <dimension ref="A1:V284"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="2" max="2" width="10.375" customWidth="1"/>
@@ -16961,6 +17027,9 @@
       <c r="E271" t="s">
         <v>217</v>
       </c>
+      <c r="F271" t="s">
+        <v>69</v>
+      </c>
       <c r="G271" s="13"/>
       <c r="H271" s="24"/>
       <c r="I271" s="24"/>
@@ -17151,52 +17220,440 @@
       </c>
     </row>
     <row r="275" spans="1:22" ht="15.75" customHeight="1">
-      <c r="A275" s="13"/>
-      <c r="B275" s="10"/>
-      <c r="C275" s="12"/>
-      <c r="D275" s="2"/>
-      <c r="E275" s="2"/>
-      <c r="F275" s="2"/>
+      <c r="A275" s="13">
+        <v>46325</v>
+      </c>
+      <c r="B275" s="10" t="s">
+        <v>393</v>
+      </c>
+      <c r="C275" s="12" t="s">
+        <v>671</v>
+      </c>
+      <c r="D275" s="2" t="s">
+        <v>672</v>
+      </c>
+      <c r="E275" t="s">
+        <v>673</v>
+      </c>
+      <c r="F275" s="2" t="s">
+        <v>69</v>
+      </c>
       <c r="G275" s="13"/>
       <c r="H275" s="24"/>
       <c r="I275" s="24"/>
       <c r="J275" s="13"/>
-      <c r="K275" s="13"/>
+      <c r="K275" s="23"/>
       <c r="L275" s="13"/>
       <c r="M275" s="24"/>
       <c r="N275" s="13"/>
-      <c r="O275" s="10"/>
-      <c r="P275" s="10"/>
-      <c r="Q275" s="10"/>
-      <c r="R275" s="10"/>
-      <c r="S275" s="10"/>
-      <c r="T275" s="10"/>
-      <c r="U275" s="10"/>
-      <c r="V275" s="6"/>
+      <c r="O275">
+        <v>0.56799999999999995</v>
+      </c>
+      <c r="P275">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="Q275" t="s">
+        <v>674</v>
+      </c>
+      <c r="R275">
+        <v>0.64</v>
+      </c>
+      <c r="S275">
+        <v>0.57799999999999996</v>
+      </c>
+      <c r="T275">
+        <v>1</v>
+      </c>
+      <c r="U275">
+        <v>0.89200000000000002</v>
+      </c>
+      <c r="V275">
+        <v>0.56200000000000006</v>
+      </c>
     </row>
     <row r="276" spans="1:22" ht="15.75" customHeight="1">
-      <c r="A276" s="13"/>
-      <c r="B276" s="10"/>
-      <c r="C276" s="12"/>
-      <c r="D276" s="2"/>
-      <c r="E276" s="2"/>
-      <c r="F276" s="2"/>
+      <c r="A276" s="13">
+        <v>46325</v>
+      </c>
+      <c r="B276" s="10" t="s">
+        <v>398</v>
+      </c>
+      <c r="C276" s="12" t="s">
+        <v>675</v>
+      </c>
+      <c r="D276" s="2" t="s">
+        <v>676</v>
+      </c>
+      <c r="E276" s="2" t="s">
+        <v>677</v>
+      </c>
+      <c r="F276" s="2" t="s">
+        <v>69</v>
+      </c>
       <c r="G276" s="13"/>
       <c r="H276" s="24"/>
       <c r="I276" s="24"/>
       <c r="J276" s="13"/>
       <c r="K276" s="13"/>
-      <c r="L276" s="13"/>
+      <c r="L276" s="23"/>
       <c r="M276" s="24"/>
       <c r="N276" s="13"/>
-      <c r="O276" s="10"/>
-      <c r="P276" s="10"/>
-      <c r="Q276" s="10"/>
-      <c r="R276" s="10"/>
-      <c r="S276" s="10"/>
-      <c r="T276" s="10"/>
-      <c r="U276" s="10"/>
-      <c r="V276" s="6"/>
+      <c r="O276">
+        <v>0.72499999999999998</v>
+      </c>
+      <c r="P276">
+        <v>0.60499999999999998</v>
+      </c>
+      <c r="Q276" t="s">
+        <v>678</v>
+      </c>
+      <c r="R276">
+        <v>0.68400000000000005</v>
+      </c>
+      <c r="S276">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="T276">
+        <v>0.94</v>
+      </c>
+      <c r="U276">
+        <v>0.84799999999999998</v>
+      </c>
+      <c r="V276">
+        <v>0.58499999999999996</v>
+      </c>
+    </row>
+    <row r="277" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A277" s="13">
+        <v>46325</v>
+      </c>
+      <c r="B277" s="10" t="s">
+        <v>393</v>
+      </c>
+      <c r="C277" s="12" t="s">
+        <v>679</v>
+      </c>
+      <c r="D277" s="2" t="s">
+        <v>481</v>
+      </c>
+      <c r="E277" s="2" t="s">
+        <v>680</v>
+      </c>
+      <c r="F277" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="G277" s="13"/>
+      <c r="H277" s="24"/>
+      <c r="I277" s="23"/>
+      <c r="J277" s="13"/>
+      <c r="K277" s="13"/>
+      <c r="L277" s="13"/>
+      <c r="M277" s="24"/>
+      <c r="N277" s="13"/>
+      <c r="O277">
+        <v>0.73499999999999999</v>
+      </c>
+      <c r="P277">
+        <v>0.65</v>
+      </c>
+      <c r="Q277" t="s">
+        <v>681</v>
+      </c>
+      <c r="R277">
+        <v>0.72</v>
+      </c>
+      <c r="S277">
+        <v>0.53900000000000003</v>
+      </c>
+      <c r="T277">
+        <v>0.96299999999999997</v>
+      </c>
+      <c r="U277">
+        <v>0.86099999999999999</v>
+      </c>
+      <c r="V277">
+        <v>0.61199999999999999</v>
+      </c>
+    </row>
+    <row r="278" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A278" s="13">
+        <v>46325</v>
+      </c>
+      <c r="B278" s="10" t="s">
+        <v>398</v>
+      </c>
+      <c r="C278" s="12" t="s">
+        <v>682</v>
+      </c>
+      <c r="D278" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="E278" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="F278" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="G278" s="13"/>
+      <c r="H278" s="24"/>
+      <c r="I278" s="24"/>
+      <c r="J278" s="13"/>
+      <c r="K278" s="13"/>
+      <c r="L278" s="23"/>
+      <c r="M278" s="24"/>
+      <c r="N278" s="13"/>
+      <c r="O278">
+        <v>0.79800000000000004</v>
+      </c>
+      <c r="P278">
+        <v>0.63700000000000001</v>
+      </c>
+      <c r="Q278" t="s">
+        <v>683</v>
+      </c>
+      <c r="R278">
+        <v>0.70899999999999996</v>
+      </c>
+      <c r="S278">
+        <v>0.54800000000000004</v>
+      </c>
+      <c r="T278">
+        <v>0.872</v>
+      </c>
+      <c r="U278">
+        <v>0.86</v>
+      </c>
+      <c r="V278">
+        <v>0.60199999999999998</v>
+      </c>
+    </row>
+    <row r="279" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A279" s="13">
+        <v>46325</v>
+      </c>
+      <c r="B279" s="10" t="s">
+        <v>393</v>
+      </c>
+      <c r="C279" t="s">
+        <v>684</v>
+      </c>
+      <c r="D279" t="s">
+        <v>578</v>
+      </c>
+      <c r="E279" t="s">
+        <v>685</v>
+      </c>
+      <c r="F279" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="G279" s="13"/>
+      <c r="H279" s="24"/>
+      <c r="I279" s="24"/>
+      <c r="J279" s="13"/>
+      <c r="K279" s="13"/>
+      <c r="L279" s="13"/>
+      <c r="M279" s="24"/>
+      <c r="N279" s="23"/>
+      <c r="O279">
+        <v>0.73</v>
+      </c>
+      <c r="P279">
+        <v>0.56799999999999995</v>
+      </c>
+      <c r="Q279" t="s">
+        <v>686</v>
+      </c>
+      <c r="R279">
+        <v>0.65400000000000003</v>
+      </c>
+      <c r="S279">
+        <v>0.57899999999999996</v>
+      </c>
+      <c r="T279">
+        <v>0.90500000000000003</v>
+      </c>
+      <c r="U279">
+        <v>0.85799999999999998</v>
+      </c>
+      <c r="V279">
+        <v>0.57899999999999996</v>
+      </c>
+    </row>
+    <row r="280" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A280" s="13">
+        <v>46325</v>
+      </c>
+      <c r="B280" s="10" t="s">
+        <v>398</v>
+      </c>
+      <c r="C280" s="12" t="s">
+        <v>687</v>
+      </c>
+      <c r="D280" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="E280" s="2" t="s">
+        <v>688</v>
+      </c>
+      <c r="F280" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="G280" s="24"/>
+      <c r="H280" s="23"/>
+      <c r="I280" s="24"/>
+      <c r="J280" s="13"/>
+      <c r="K280" s="13"/>
+      <c r="L280" s="13"/>
+      <c r="M280" s="24"/>
+      <c r="N280" s="13"/>
+      <c r="O280">
+        <v>0.626</v>
+      </c>
+      <c r="P280">
+        <v>0.65800000000000003</v>
+      </c>
+      <c r="Q280" t="s">
+        <v>689</v>
+      </c>
+      <c r="R280">
+        <v>0.72699999999999998</v>
+      </c>
+      <c r="S280">
+        <v>0.54</v>
+      </c>
+      <c r="T280">
+        <v>0.74</v>
+      </c>
+      <c r="U280">
+        <v>0.88800000000000001</v>
+      </c>
+      <c r="V280">
+        <v>0.56399999999999995</v>
+      </c>
+    </row>
+    <row r="281" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A281" s="13">
+        <v>46325</v>
+      </c>
+      <c r="B281" s="10" t="s">
+        <v>393</v>
+      </c>
+      <c r="C281" t="s">
+        <v>690</v>
+      </c>
+      <c r="D281" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="E281" s="2" t="s">
+        <v>691</v>
+      </c>
+      <c r="F281" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="G281" s="13"/>
+      <c r="H281" s="24"/>
+      <c r="I281" s="24"/>
+      <c r="J281" s="13"/>
+      <c r="K281" s="13"/>
+      <c r="L281" s="23"/>
+      <c r="M281" s="24"/>
+      <c r="N281" s="13"/>
+      <c r="O281">
+        <v>0.72599999999999998</v>
+      </c>
+      <c r="P281">
+        <v>0.63800000000000001</v>
+      </c>
+      <c r="Q281" t="s">
+        <v>692</v>
+      </c>
+      <c r="R281">
+        <v>0.71</v>
+      </c>
+      <c r="S281">
+        <v>0.54900000000000004</v>
+      </c>
+      <c r="T281">
+        <v>0.91</v>
+      </c>
+      <c r="U281">
+        <v>0.83799999999999997</v>
+      </c>
+      <c r="V281">
+        <v>0.59</v>
+      </c>
+    </row>
+    <row r="282" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A282" s="13"/>
+      <c r="B282" s="10"/>
+      <c r="C282" s="12"/>
+      <c r="D282" s="2"/>
+      <c r="E282" s="2"/>
+      <c r="F282" s="2"/>
+      <c r="G282" s="13"/>
+      <c r="H282" s="24"/>
+      <c r="I282" s="24"/>
+      <c r="J282" s="13"/>
+      <c r="K282" s="13"/>
+      <c r="L282" s="13"/>
+      <c r="M282" s="24"/>
+      <c r="N282" s="13"/>
+      <c r="O282" s="10"/>
+      <c r="P282" s="10"/>
+      <c r="Q282" s="10"/>
+      <c r="R282" s="10"/>
+      <c r="S282" s="10"/>
+      <c r="T282" s="10"/>
+      <c r="U282" s="10"/>
+      <c r="V282" s="6"/>
+    </row>
+    <row r="283" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A283" s="13"/>
+      <c r="B283" s="10"/>
+      <c r="C283" s="12"/>
+      <c r="D283" s="2"/>
+      <c r="E283" s="2"/>
+      <c r="F283" s="2"/>
+      <c r="G283" s="13"/>
+      <c r="H283" s="24"/>
+      <c r="I283" s="24"/>
+      <c r="J283" s="13"/>
+      <c r="K283" s="13"/>
+      <c r="L283" s="13"/>
+      <c r="M283" s="24"/>
+      <c r="N283" s="13"/>
+      <c r="O283" s="10"/>
+      <c r="P283" s="10"/>
+      <c r="Q283" s="10"/>
+      <c r="R283" s="10"/>
+      <c r="S283" s="10"/>
+      <c r="T283" s="10"/>
+      <c r="U283" s="10"/>
+      <c r="V283" s="6"/>
+    </row>
+    <row r="284" spans="1:22" ht="15.75" customHeight="1">
+      <c r="A284" s="13"/>
+      <c r="B284" s="10"/>
+      <c r="C284" s="12"/>
+      <c r="D284" s="2"/>
+      <c r="E284" s="2"/>
+      <c r="F284" s="2"/>
+      <c r="G284" s="13"/>
+      <c r="H284" s="24"/>
+      <c r="I284" s="24"/>
+      <c r="J284" s="13"/>
+      <c r="K284" s="13"/>
+      <c r="L284" s="13"/>
+      <c r="M284" s="24"/>
+      <c r="N284" s="13"/>
+      <c r="O284" s="10"/>
+      <c r="P284" s="10"/>
+      <c r="Q284" s="10"/>
+      <c r="R284" s="10"/>
+      <c r="S284" s="10"/>
+      <c r="T284" s="10"/>
+      <c r="U284" s="10"/>
+      <c r="V284" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>